<commit_message>
Reformat contact number according to country of origin
</commit_message>
<xml_diff>
--- a/10k_adhoc_leads/Merged_Raw_Data/Merge_Kalai_and_Ish/Merged_F&B_Prospects_from_Ishwarya's_Own.xlsx
+++ b/10k_adhoc_leads/Merged_Raw_Data/Merge_Kalai_and_Ish/Merged_F&B_Prospects_from_Ishwarya's_Own.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1615"/>
+  <dimension ref="A1:E1593"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28477,29 +28477,31 @@
     <row r="1385">
       <c r="A1385" t="inlineStr">
         <is>
-          <t>A Noodle Story</t>
+          <t>Aburiyatei</t>
         </is>
       </c>
       <c r="B1385" t="inlineStr"/>
       <c r="C1385" t="inlineStr">
         <is>
-          <t>#ERROR!</t>
-        </is>
-      </c>
-      <c r="D1385" t="inlineStr"/>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1385" t="inlineStr"/>
     </row>
     <row r="1386">
       <c r="A1386" t="inlineStr">
         <is>
-          <t>Absinthe</t>
+          <t>Adam's seafood corner</t>
         </is>
       </c>
       <c r="B1386" t="inlineStr"/>
-      <c r="C1386" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1386" t="n">
+        <v>62941821</v>
       </c>
       <c r="D1386" t="inlineStr"/>
       <c r="E1386" t="inlineStr"/>
@@ -28507,44 +28509,44 @@
     <row r="1387">
       <c r="A1387" t="inlineStr">
         <is>
-          <t>Aburiyatei</t>
+          <t>Adonis Hotel</t>
         </is>
       </c>
       <c r="B1387" t="inlineStr"/>
-      <c r="C1387" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1387" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1387" t="n">
+        <v>63360013</v>
+      </c>
+      <c r="D1387" t="inlineStr"/>
       <c r="E1387" t="inlineStr"/>
     </row>
     <row r="1388">
       <c r="A1388" t="inlineStr">
         <is>
-          <t>Adam's seafood corner</t>
+          <t>Ah Yat Abalone Forum Restaurant</t>
         </is>
       </c>
       <c r="B1388" t="inlineStr"/>
-      <c r="C1388" t="n">
-        <v>62941821</v>
-      </c>
-      <c r="D1388" t="inlineStr"/>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1388" t="inlineStr"/>
     </row>
     <row r="1389">
       <c r="A1389" t="inlineStr">
         <is>
-          <t>Adonis Hotel</t>
+          <t>Al Hamra Lebanese &amp; Middle Eastern Restaurant</t>
         </is>
       </c>
       <c r="B1389" t="inlineStr"/>
       <c r="C1389" t="n">
-        <v>63360013</v>
+        <v>64648488</v>
       </c>
       <c r="D1389" t="inlineStr"/>
       <c r="E1389" t="inlineStr"/>
@@ -28552,31 +28554,27 @@
     <row r="1390">
       <c r="A1390" t="inlineStr">
         <is>
-          <t>Ah Yat Abalone Forum Restaurant</t>
+          <t>Amravati Andhra Kuchullu</t>
         </is>
       </c>
       <c r="B1390" t="inlineStr"/>
-      <c r="C1390" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1390" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1390" t="n">
+        <v>82803061</v>
+      </c>
+      <c r="D1390" t="inlineStr"/>
       <c r="E1390" t="inlineStr"/>
     </row>
     <row r="1391">
       <c r="A1391" t="inlineStr">
         <is>
-          <t>Al Hamra Lebanese &amp; Middle Eastern Restaurant</t>
+          <t>Ananas Café</t>
         </is>
       </c>
       <c r="B1391" t="inlineStr"/>
-      <c r="C1391" t="n">
-        <v>64648488</v>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>(+65) 9800 5633</t>
+        </is>
       </c>
       <c r="D1391" t="inlineStr"/>
       <c r="E1391" t="inlineStr"/>
@@ -28584,12 +28582,14 @@
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
-          <t>Amravati Andhra Kuchullu</t>
+          <t>Ananda Bhavan deal</t>
         </is>
       </c>
       <c r="B1392" t="inlineStr"/>
-      <c r="C1392" t="n">
-        <v>82803061</v>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>6299 4466</t>
+        </is>
       </c>
       <c r="D1392" t="inlineStr"/>
       <c r="E1392" t="inlineStr"/>
@@ -28597,14 +28597,12 @@
     <row r="1393">
       <c r="A1393" t="inlineStr">
         <is>
-          <t>Ananas Café</t>
+          <t>Anatolia Turkish Restaurant</t>
         </is>
       </c>
       <c r="B1393" t="inlineStr"/>
-      <c r="C1393" t="inlineStr">
-        <is>
-          <t>(+65) 9800 5633</t>
-        </is>
+      <c r="C1393" t="n">
+        <v>68363352</v>
       </c>
       <c r="D1393" t="inlineStr"/>
       <c r="E1393" t="inlineStr"/>
@@ -28612,14 +28610,12 @@
     <row r="1394">
       <c r="A1394" t="inlineStr">
         <is>
-          <t>Ananda Bhavan deal</t>
+          <t>And All Things Delicious</t>
         </is>
       </c>
       <c r="B1394" t="inlineStr"/>
-      <c r="C1394" t="inlineStr">
-        <is>
-          <t>6299 4466</t>
-        </is>
+      <c r="C1394" t="n">
+        <v>62914252</v>
       </c>
       <c r="D1394" t="inlineStr"/>
       <c r="E1394" t="inlineStr"/>
@@ -28627,25 +28623,31 @@
     <row r="1395">
       <c r="A1395" t="inlineStr">
         <is>
-          <t>Anatolia Turkish Restaurant</t>
+          <t>Andersen's Of Denmark Ice Cream</t>
         </is>
       </c>
       <c r="B1395" t="inlineStr"/>
-      <c r="C1395" t="n">
-        <v>68363352</v>
-      </c>
-      <c r="D1395" t="inlineStr"/>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>68469555 (O)</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6634 2308</t>
+        </is>
+      </c>
       <c r="E1395" t="inlineStr"/>
     </row>
     <row r="1396">
       <c r="A1396" t="inlineStr">
         <is>
-          <t>And All Things Delicious</t>
+          <t>Andhra Curry</t>
         </is>
       </c>
       <c r="B1396" t="inlineStr"/>
       <c r="C1396" t="n">
-        <v>62914252</v>
+        <v>81219993</v>
       </c>
       <c r="D1396" t="inlineStr"/>
       <c r="E1396" t="inlineStr"/>
@@ -28653,18 +28655,18 @@
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
-          <t>Andersen's Of Denmark Ice Cream</t>
+          <t>Appare Japanese Restaurant</t>
         </is>
       </c>
       <c r="B1397" t="inlineStr"/>
       <c r="C1397" t="inlineStr">
         <is>
-          <t>68469555 (O)</t>
+          <t>6227 0331</t>
         </is>
       </c>
       <c r="D1397" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6634 2308</t>
+          <t xml:space="preserve"> 6532 9006</t>
         </is>
       </c>
       <c r="E1397" t="inlineStr"/>
@@ -28672,63 +28674,57 @@
     <row r="1398">
       <c r="A1398" t="inlineStr">
         <is>
-          <t>Andhra Curry</t>
+          <t>Apples &amp; Oranges</t>
         </is>
       </c>
       <c r="B1398" t="inlineStr"/>
-      <c r="C1398" t="n">
-        <v>81219993</v>
-      </c>
-      <c r="D1398" t="inlineStr"/>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1398" t="inlineStr"/>
     </row>
     <row r="1399">
       <c r="A1399" t="inlineStr">
         <is>
-          <t>Appare Japanese Restaurant</t>
+          <t>Appu's Curry</t>
         </is>
       </c>
       <c r="B1399" t="inlineStr"/>
-      <c r="C1399" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1399" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1399" t="n">
+        <v>62911629</v>
+      </c>
+      <c r="D1399" t="inlineStr"/>
       <c r="E1399" t="inlineStr"/>
     </row>
     <row r="1400">
       <c r="A1400" t="inlineStr">
         <is>
-          <t>Apples &amp; Oranges</t>
+          <t>Aqua Luna</t>
         </is>
       </c>
       <c r="B1400" t="inlineStr"/>
-      <c r="C1400" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1400" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1400" t="n">
+        <v>68288888</v>
+      </c>
+      <c r="D1400" t="inlineStr"/>
       <c r="E1400" t="inlineStr"/>
     </row>
     <row r="1401">
       <c r="A1401" t="inlineStr">
         <is>
-          <t>Appu's Curry</t>
+          <t>Arashi Yakiniku Charcoal Grill Restaurant</t>
         </is>
       </c>
       <c r="B1401" t="inlineStr"/>
       <c r="C1401" t="n">
-        <v>62911629</v>
+        <v>62651004</v>
       </c>
       <c r="D1401" t="inlineStr"/>
       <c r="E1401" t="inlineStr"/>
@@ -28736,12 +28732,12 @@
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
-          <t>Aqua Luna</t>
+          <t>Aravind's Curry</t>
         </is>
       </c>
       <c r="B1402" t="inlineStr"/>
       <c r="C1402" t="n">
-        <v>68288888</v>
+        <v>62988933</v>
       </c>
       <c r="D1402" t="inlineStr"/>
       <c r="E1402" t="inlineStr"/>
@@ -28749,12 +28745,12 @@
     <row r="1403">
       <c r="A1403" t="inlineStr">
         <is>
-          <t>Arashi Yakiniku Charcoal Grill Restaurant</t>
+          <t>Aranda Lounge</t>
         </is>
       </c>
       <c r="B1403" t="inlineStr"/>
       <c r="C1403" t="n">
-        <v>62651004</v>
+        <v>67559811</v>
       </c>
       <c r="D1403" t="inlineStr"/>
       <c r="E1403" t="inlineStr"/>
@@ -28762,25 +28758,29 @@
     <row r="1404">
       <c r="A1404" t="inlineStr">
         <is>
-          <t>Aravind's Curry</t>
+          <t>Aromas Of India</t>
         </is>
       </c>
       <c r="B1404" t="inlineStr"/>
       <c r="C1404" t="n">
-        <v>62988933</v>
-      </c>
-      <c r="D1404" t="inlineStr"/>
+        <v>62562448</v>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6256 2448</t>
+        </is>
+      </c>
       <c r="E1404" t="inlineStr"/>
     </row>
     <row r="1405">
       <c r="A1405" t="inlineStr">
         <is>
-          <t>Aranda Lounge</t>
+          <t>Arteastiq Group *</t>
         </is>
       </c>
       <c r="B1405" t="inlineStr"/>
       <c r="C1405" t="n">
-        <v>67559811</v>
+        <v>62358370</v>
       </c>
       <c r="D1405" t="inlineStr"/>
       <c r="E1405" t="inlineStr"/>
@@ -28788,29 +28788,25 @@
     <row r="1406">
       <c r="A1406" t="inlineStr">
         <is>
-          <t>Aromas Of India</t>
+          <t>Artemis Grill</t>
         </is>
       </c>
       <c r="B1406" t="inlineStr"/>
       <c r="C1406" t="n">
-        <v>62562448</v>
-      </c>
-      <c r="D1406" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6256 2448</t>
-        </is>
-      </c>
+        <v>66358677</v>
+      </c>
+      <c r="D1406" t="inlineStr"/>
       <c r="E1406" t="inlineStr"/>
     </row>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
-          <t>Arteastiq Group *</t>
+          <t>Ashino</t>
         </is>
       </c>
       <c r="B1407" t="inlineStr"/>
       <c r="C1407" t="n">
-        <v>62358370</v>
+        <v>66844567</v>
       </c>
       <c r="D1407" t="inlineStr"/>
       <c r="E1407" t="inlineStr"/>
@@ -28818,12 +28814,12 @@
     <row r="1408">
       <c r="A1408" t="inlineStr">
         <is>
-          <t>Artemis Grill</t>
+          <t>Asian Halalfood Pte. Ltd.</t>
         </is>
       </c>
       <c r="B1408" t="inlineStr"/>
       <c r="C1408" t="n">
-        <v>66358677</v>
+        <v>62616887</v>
       </c>
       <c r="D1408" t="inlineStr"/>
       <c r="E1408" t="inlineStr"/>
@@ -28831,29 +28827,27 @@
     <row r="1409">
       <c r="A1409" t="inlineStr">
         <is>
-          <t>Artistry Cafe deal</t>
+          <t>Assembly Coffee</t>
         </is>
       </c>
       <c r="B1409" t="inlineStr"/>
-      <c r="C1409" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
-      </c>
-      <c r="D1409" t="inlineStr"/>
+      <c r="C1409" t="n">
+        <v>67355647</v>
+      </c>
+      <c r="D1409" t="n">
+        <v>67333375</v>
+      </c>
       <c r="E1409" t="inlineStr"/>
     </row>
     <row r="1410">
       <c r="A1410" t="inlineStr">
         <is>
-          <t>Artichoke deal</t>
+          <t>Attica Bar</t>
         </is>
       </c>
       <c r="B1410" t="inlineStr"/>
-      <c r="C1410" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1410" t="n">
+        <v>63339973</v>
       </c>
       <c r="D1410" t="inlineStr"/>
       <c r="E1410" t="inlineStr"/>
@@ -28861,12 +28855,14 @@
     <row r="1411">
       <c r="A1411" t="inlineStr">
         <is>
-          <t>Ashino</t>
+          <t>Auntie Kim's Korean Restaurant</t>
         </is>
       </c>
       <c r="B1411" t="inlineStr"/>
-      <c r="C1411" t="n">
-        <v>66844567</v>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>6452-2112 Thomson</t>
+        </is>
       </c>
       <c r="D1411" t="inlineStr"/>
       <c r="E1411" t="inlineStr"/>
@@ -28874,40 +28870,40 @@
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
-          <t>Asian Halalfood Pte. Ltd.</t>
+          <t>Club Aura deal</t>
         </is>
       </c>
       <c r="B1412" t="inlineStr"/>
       <c r="C1412" t="n">
-        <v>62616887</v>
-      </c>
-      <c r="D1412" t="inlineStr"/>
+        <v>68661977</v>
+      </c>
+      <c r="D1412" t="n">
+        <v>68661978</v>
+      </c>
       <c r="E1412" t="inlineStr"/>
     </row>
     <row r="1413">
       <c r="A1413" t="inlineStr">
         <is>
-          <t>Assembly Coffee</t>
+          <t>Avenue Joffre</t>
         </is>
       </c>
       <c r="B1413" t="inlineStr"/>
       <c r="C1413" t="n">
-        <v>67355647</v>
-      </c>
-      <c r="D1413" t="n">
-        <v>67333375</v>
-      </c>
+        <v>65703213</v>
+      </c>
+      <c r="D1413" t="inlineStr"/>
       <c r="E1413" t="inlineStr"/>
     </row>
     <row r="1414">
       <c r="A1414" t="inlineStr">
         <is>
-          <t>Attica Bar</t>
+          <t>Ayam Bakar Ojolali</t>
         </is>
       </c>
       <c r="B1414" t="inlineStr"/>
       <c r="C1414" t="n">
-        <v>63339973</v>
+        <v>91732779</v>
       </c>
       <c r="D1414" t="inlineStr"/>
       <c r="E1414" t="inlineStr"/>
@@ -28915,14 +28911,12 @@
     <row r="1415">
       <c r="A1415" t="inlineStr">
         <is>
-          <t>Au Petit Salut</t>
+          <t>Azzura Resorts Pte. Ltd.</t>
         </is>
       </c>
       <c r="B1415" t="inlineStr"/>
-      <c r="C1415" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1415" t="n">
+        <v>62708003</v>
       </c>
       <c r="D1415" t="inlineStr"/>
       <c r="E1415" t="inlineStr"/>
@@ -28930,14 +28924,12 @@
     <row r="1416">
       <c r="A1416" t="inlineStr">
         <is>
-          <t>Auntie Kim's Korean Restaurant</t>
+          <t>B @ Rochester</t>
         </is>
       </c>
       <c r="B1416" t="inlineStr"/>
-      <c r="C1416" t="inlineStr">
-        <is>
-          <t>6452-2112 Thomson</t>
-        </is>
+      <c r="C1416" t="n">
+        <v>67781788</v>
       </c>
       <c r="D1416" t="inlineStr"/>
       <c r="E1416" t="inlineStr"/>
@@ -28945,27 +28937,27 @@
     <row r="1417">
       <c r="A1417" t="inlineStr">
         <is>
-          <t>Club Aura deal</t>
+          <t>Ba.Li.Ba. Pub &amp; Cafe</t>
         </is>
       </c>
       <c r="B1417" t="inlineStr"/>
       <c r="C1417" t="n">
-        <v>68661977</v>
+        <v>67362056</v>
       </c>
       <c r="D1417" t="n">
-        <v>68661978</v>
+        <v>67376036</v>
       </c>
       <c r="E1417" t="inlineStr"/>
     </row>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
-          <t>Avenue Joffre</t>
+          <t>Back Benchers Cafe &amp; Bar</t>
         </is>
       </c>
       <c r="B1418" t="inlineStr"/>
       <c r="C1418" t="n">
-        <v>65703213</v>
+        <v>62210150</v>
       </c>
       <c r="D1418" t="inlineStr"/>
       <c r="E1418" t="inlineStr"/>
@@ -28973,12 +28965,12 @@
     <row r="1419">
       <c r="A1419" t="inlineStr">
         <is>
-          <t>Ayam Bakar Ojolali</t>
+          <t>BACON &amp; BOOZE</t>
         </is>
       </c>
       <c r="B1419" t="inlineStr"/>
       <c r="C1419" t="n">
-        <v>91732779</v>
+        <v>64895679</v>
       </c>
       <c r="D1419" t="inlineStr"/>
       <c r="E1419" t="inlineStr"/>
@@ -28986,12 +28978,12 @@
     <row r="1420">
       <c r="A1420" t="inlineStr">
         <is>
-          <t>Azzura Resorts Pte. Ltd.</t>
+          <t>Baja Fresh</t>
         </is>
       </c>
       <c r="B1420" t="inlineStr"/>
       <c r="C1420" t="n">
-        <v>62708003</v>
+        <v>81574136</v>
       </c>
       <c r="D1420" t="inlineStr"/>
       <c r="E1420" t="inlineStr"/>
@@ -28999,12 +28991,12 @@
     <row r="1421">
       <c r="A1421" t="inlineStr">
         <is>
-          <t>B @ Rochester</t>
+          <t>Badoque Cafe</t>
         </is>
       </c>
       <c r="B1421" t="inlineStr"/>
       <c r="C1421" t="n">
-        <v>67781788</v>
+        <v>64466928</v>
       </c>
       <c r="D1421" t="inlineStr"/>
       <c r="E1421" t="inlineStr"/>
@@ -29012,27 +29004,25 @@
     <row r="1422">
       <c r="A1422" t="inlineStr">
         <is>
-          <t>Ba.Li.Ba. Pub &amp; Cafe</t>
+          <t>Balaji Bhawan</t>
         </is>
       </c>
       <c r="B1422" t="inlineStr"/>
       <c r="C1422" t="n">
-        <v>67362056</v>
-      </c>
-      <c r="D1422" t="n">
-        <v>67376036</v>
-      </c>
+        <v>91267797</v>
+      </c>
+      <c r="D1422" t="inlineStr"/>
       <c r="E1422" t="inlineStr"/>
     </row>
     <row r="1423">
       <c r="A1423" t="inlineStr">
         <is>
-          <t>Back Benchers Cafe &amp; Bar</t>
+          <t>Balaclava (SG)</t>
         </is>
       </c>
       <c r="B1423" t="inlineStr"/>
       <c r="C1423" t="n">
-        <v>62210150</v>
+        <v>63360050</v>
       </c>
       <c r="D1423" t="inlineStr"/>
       <c r="E1423" t="inlineStr"/>
@@ -29040,14 +29030,12 @@
     <row r="1424">
       <c r="A1424" t="inlineStr">
         <is>
-          <t>Baci Baci</t>
+          <t>Balance Delight Coffeeshop</t>
         </is>
       </c>
       <c r="B1424" t="inlineStr"/>
-      <c r="C1424" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1424" t="n">
+        <v>83633340</v>
       </c>
       <c r="D1424" t="inlineStr"/>
       <c r="E1424" t="inlineStr"/>
@@ -29055,12 +29043,12 @@
     <row r="1425">
       <c r="A1425" t="inlineStr">
         <is>
-          <t>BACON &amp; BOOZE</t>
+          <t>Balzac Brasserie &amp; Bar</t>
         </is>
       </c>
       <c r="B1425" t="inlineStr"/>
       <c r="C1425" t="n">
-        <v>64895679</v>
+        <v>63360797</v>
       </c>
       <c r="D1425" t="inlineStr"/>
       <c r="E1425" t="inlineStr"/>
@@ -29068,12 +29056,12 @@
     <row r="1426">
       <c r="A1426" t="inlineStr">
         <is>
-          <t>Baja Fresh</t>
+          <t>Bam! Tapas Sake Bar</t>
         </is>
       </c>
       <c r="B1426" t="inlineStr"/>
       <c r="C1426" t="n">
-        <v>81574136</v>
+        <v>62260500</v>
       </c>
       <c r="D1426" t="inlineStr"/>
       <c r="E1426" t="inlineStr"/>
@@ -29081,14 +29069,12 @@
     <row r="1427">
       <c r="A1427" t="inlineStr">
         <is>
-          <t>Bakers Well</t>
+          <t>Baquette</t>
         </is>
       </c>
       <c r="B1427" t="inlineStr"/>
-      <c r="C1427" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1427" t="n">
+        <v>97367480</v>
       </c>
       <c r="D1427" t="inlineStr"/>
       <c r="E1427" t="inlineStr"/>
@@ -29096,12 +29082,12 @@
     <row r="1428">
       <c r="A1428" t="inlineStr">
         <is>
-          <t>Badoque Cafe</t>
+          <t>Bar A Vin</t>
         </is>
       </c>
       <c r="B1428" t="inlineStr"/>
       <c r="C1428" t="n">
-        <v>64466928</v>
+        <v>64389982</v>
       </c>
       <c r="D1428" t="inlineStr"/>
       <c r="E1428" t="inlineStr"/>
@@ -29109,12 +29095,12 @@
     <row r="1429">
       <c r="A1429" t="inlineStr">
         <is>
-          <t>Balaji Bhawan</t>
+          <t>Bar.B.Q Tonight Restaurant</t>
         </is>
       </c>
       <c r="B1429" t="inlineStr"/>
       <c r="C1429" t="n">
-        <v>91267797</v>
+        <v>63279280</v>
       </c>
       <c r="D1429" t="inlineStr"/>
       <c r="E1429" t="inlineStr"/>
@@ -29122,12 +29108,12 @@
     <row r="1430">
       <c r="A1430" t="inlineStr">
         <is>
-          <t>Balaclava (SG)</t>
+          <t>Bar Canary</t>
         </is>
       </c>
       <c r="B1430" t="inlineStr"/>
       <c r="C1430" t="n">
-        <v>63360050</v>
+        <v>66038855</v>
       </c>
       <c r="D1430" t="inlineStr"/>
       <c r="E1430" t="inlineStr"/>
@@ -29135,12 +29121,12 @@
     <row r="1431">
       <c r="A1431" t="inlineStr">
         <is>
-          <t>Balance Delight Coffeeshop</t>
+          <t>Barpazza</t>
         </is>
       </c>
       <c r="B1431" t="inlineStr"/>
       <c r="C1431" t="n">
-        <v>83633340</v>
+        <v>65360572</v>
       </c>
       <c r="D1431" t="inlineStr"/>
       <c r="E1431" t="inlineStr"/>
@@ -29148,12 +29134,12 @@
     <row r="1432">
       <c r="A1432" t="inlineStr">
         <is>
-          <t>Balzac Brasserie &amp; Bar</t>
+          <t>BarRoque Grill</t>
         </is>
       </c>
       <c r="B1432" t="inlineStr"/>
       <c r="C1432" t="n">
-        <v>63360797</v>
+        <v>64449672</v>
       </c>
       <c r="D1432" t="inlineStr"/>
       <c r="E1432" t="inlineStr"/>
@@ -29161,12 +29147,12 @@
     <row r="1433">
       <c r="A1433" t="inlineStr">
         <is>
-          <t>Bam! Tapas Sake Bar</t>
+          <t>Basilico @ Regent Singapore</t>
         </is>
       </c>
       <c r="B1433" t="inlineStr"/>
       <c r="C1433" t="n">
-        <v>62260500</v>
+        <v>67323202</v>
       </c>
       <c r="D1433" t="inlineStr"/>
       <c r="E1433" t="inlineStr"/>
@@ -29174,12 +29160,12 @@
     <row r="1434">
       <c r="A1434" t="inlineStr">
         <is>
-          <t>Baquette</t>
+          <t>BayView Tandoor</t>
         </is>
       </c>
       <c r="B1434" t="inlineStr"/>
       <c r="C1434" t="n">
-        <v>97367480</v>
+        <v>98621981</v>
       </c>
       <c r="D1434" t="inlineStr"/>
       <c r="E1434" t="inlineStr"/>
@@ -29187,12 +29173,12 @@
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
-          <t>Bar A Vin</t>
+          <t>Bearbites cafe</t>
         </is>
       </c>
       <c r="B1435" t="inlineStr"/>
       <c r="C1435" t="n">
-        <v>64389982</v>
+        <v>90255121</v>
       </c>
       <c r="D1435" t="inlineStr"/>
       <c r="E1435" t="inlineStr"/>
@@ -29200,12 +29186,12 @@
     <row r="1436">
       <c r="A1436" t="inlineStr">
         <is>
-          <t>Bar.B.Q Tonight Restaurant</t>
+          <t>BBQ World Korean Restaurant</t>
         </is>
       </c>
       <c r="B1436" t="inlineStr"/>
       <c r="C1436" t="n">
-        <v>63279280</v>
+        <v>63245017</v>
       </c>
       <c r="D1436" t="inlineStr"/>
       <c r="E1436" t="inlineStr"/>
@@ -29213,12 +29199,12 @@
     <row r="1437">
       <c r="A1437" t="inlineStr">
         <is>
-          <t>Bar Canary</t>
+          <t>Bee kee wanton noodles</t>
         </is>
       </c>
       <c r="B1437" t="inlineStr"/>
       <c r="C1437" t="n">
-        <v>66038855</v>
+        <v>98773310</v>
       </c>
       <c r="D1437" t="inlineStr"/>
       <c r="E1437" t="inlineStr"/>
@@ -29226,12 +29212,12 @@
     <row r="1438">
       <c r="A1438" t="inlineStr">
         <is>
-          <t>Barpazza</t>
+          <t>Beijing Neng Ren Ju</t>
         </is>
       </c>
       <c r="B1438" t="inlineStr"/>
       <c r="C1438" t="n">
-        <v>65360572</v>
+        <v>68448553</v>
       </c>
       <c r="D1438" t="inlineStr"/>
       <c r="E1438" t="inlineStr"/>
@@ -29239,12 +29225,12 @@
     <row r="1439">
       <c r="A1439" t="inlineStr">
         <is>
-          <t>BarRoque Grill</t>
+          <t>Beer Brisket Wings</t>
         </is>
       </c>
       <c r="B1439" t="inlineStr"/>
       <c r="C1439" t="n">
-        <v>64449672</v>
+        <v>82339810</v>
       </c>
       <c r="D1439" t="inlineStr"/>
       <c r="E1439" t="inlineStr"/>
@@ -29252,12 +29238,12 @@
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
-          <t>Basilico @ Regent Singapore</t>
+          <t>ARIA| Food. Music. Arts.</t>
         </is>
       </c>
       <c r="B1440" t="inlineStr"/>
       <c r="C1440" t="n">
-        <v>67323202</v>
+        <v>63840854</v>
       </c>
       <c r="D1440" t="inlineStr"/>
       <c r="E1440" t="inlineStr"/>
@@ -29265,14 +29251,12 @@
     <row r="1441">
       <c r="A1441" t="inlineStr">
         <is>
-          <t>Basil Leaf</t>
+          <t>Arossa Wine &amp; Grill</t>
         </is>
       </c>
       <c r="B1441" t="inlineStr"/>
-      <c r="C1441" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1441" t="n">
+        <v>66362951</v>
       </c>
       <c r="D1441" t="inlineStr"/>
       <c r="E1441" t="inlineStr"/>
@@ -29280,12 +29264,12 @@
     <row r="1442">
       <c r="A1442" t="inlineStr">
         <is>
-          <t>BayView Tandoor</t>
+          <t>Aroy-dee Thai Kitchen</t>
         </is>
       </c>
       <c r="B1442" t="inlineStr"/>
       <c r="C1442" t="n">
-        <v>98621981</v>
+        <v>66352698</v>
       </c>
       <c r="D1442" t="inlineStr"/>
       <c r="E1442" t="inlineStr"/>
@@ -29293,39 +29277,51 @@
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
-          <t>Bearbites cafe</t>
+          <t>Art Pastry (CJS) at ADM</t>
         </is>
       </c>
       <c r="B1443" t="inlineStr"/>
-      <c r="C1443" t="n">
-        <v>90255121</v>
-      </c>
-      <c r="D1443" t="inlineStr"/>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1443" t="inlineStr"/>
     </row>
     <row r="1444">
       <c r="A1444" t="inlineStr">
         <is>
-          <t>BBQ World Korean Restaurant</t>
+          <t>Artisan C. Speciality Coffee</t>
         </is>
       </c>
       <c r="B1444" t="inlineStr"/>
-      <c r="C1444" t="n">
-        <v>63245017</v>
-      </c>
-      <c r="D1444" t="inlineStr"/>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1444" t="inlineStr"/>
     </row>
     <row r="1445">
       <c r="A1445" t="inlineStr">
         <is>
-          <t>Beaujolais Bar</t>
+          <t>Asian Market Café</t>
         </is>
       </c>
       <c r="B1445" t="inlineStr"/>
       <c r="C1445" t="inlineStr">
         <is>
-          <t>#ERROR!</t>
+          <t>6431 6156</t>
         </is>
       </c>
       <c r="D1445" t="inlineStr"/>
@@ -29334,12 +29330,12 @@
     <row r="1446">
       <c r="A1446" t="inlineStr">
         <is>
-          <t>Bee kee wanton noodles</t>
+          <t>Atmosphere Bistro &amp; Bar deal</t>
         </is>
       </c>
       <c r="B1446" t="inlineStr"/>
       <c r="C1446" t="n">
-        <v>98773310</v>
+        <v>67024906</v>
       </c>
       <c r="D1446" t="inlineStr"/>
       <c r="E1446" t="inlineStr"/>
@@ -29347,12 +29343,12 @@
     <row r="1447">
       <c r="A1447" t="inlineStr">
         <is>
-          <t>Beijing Neng Ren Ju</t>
+          <t>Awe desserts</t>
         </is>
       </c>
       <c r="B1447" t="inlineStr"/>
       <c r="C1447" t="n">
-        <v>68448553</v>
+        <v>63377430</v>
       </c>
       <c r="D1447" t="inlineStr"/>
       <c r="E1447" t="inlineStr"/>
@@ -29360,12 +29356,12 @@
     <row r="1448">
       <c r="A1448" t="inlineStr">
         <is>
-          <t>Beer Brisket Wings</t>
+          <t>Azabu Sabo</t>
         </is>
       </c>
       <c r="B1448" t="inlineStr"/>
       <c r="C1448" t="n">
-        <v>82339810</v>
+        <v>94235594</v>
       </c>
       <c r="D1448" t="inlineStr"/>
       <c r="E1448" t="inlineStr"/>
@@ -29373,12 +29369,14 @@
     <row r="1449">
       <c r="A1449" t="inlineStr">
         <is>
-          <t>ARIA| Food. Music. Arts.</t>
+          <t>Azmi restaurant</t>
         </is>
       </c>
       <c r="B1449" t="inlineStr"/>
-      <c r="C1449" t="n">
-        <v>63840854</v>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>9428 0203</t>
+        </is>
       </c>
       <c r="D1449" t="inlineStr"/>
       <c r="E1449" t="inlineStr"/>
@@ -29386,25 +29384,31 @@
     <row r="1450">
       <c r="A1450" t="inlineStr">
         <is>
-          <t>Arossa Wine &amp; Grill</t>
+          <t>Bangrak Thai Kitchen</t>
         </is>
       </c>
       <c r="B1450" t="inlineStr"/>
-      <c r="C1450" t="n">
-        <v>66362951</v>
-      </c>
-      <c r="D1450" t="inlineStr"/>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1450" t="inlineStr"/>
     </row>
     <row r="1451">
       <c r="A1451" t="inlineStr">
         <is>
-          <t>Aroy-dee Thai Kitchen</t>
+          <t>Bao Today</t>
         </is>
       </c>
       <c r="B1451" t="inlineStr"/>
       <c r="C1451" t="n">
-        <v>66352698</v>
+        <v>62521074</v>
       </c>
       <c r="D1451" t="inlineStr"/>
       <c r="E1451" t="inlineStr"/>
@@ -29412,52 +29416,38 @@
     <row r="1452">
       <c r="A1452" t="inlineStr">
         <is>
-          <t>Art Pastry (CJS) at ADM</t>
+          <t>Bar-a-Thym</t>
         </is>
       </c>
       <c r="B1452" t="inlineStr"/>
-      <c r="C1452" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1452" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1452" t="n">
+        <v>65572224</v>
+      </c>
+      <c r="D1452" t="inlineStr"/>
       <c r="E1452" t="inlineStr"/>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
         <is>
-          <t>Artisan C. Speciality Coffee</t>
+          <t>Barcook Bakery</t>
         </is>
       </c>
       <c r="B1453" t="inlineStr"/>
-      <c r="C1453" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1453" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1453" t="n">
+        <v>64626588</v>
+      </c>
+      <c r="D1453" t="inlineStr"/>
       <c r="E1453" t="inlineStr"/>
     </row>
     <row r="1454">
       <c r="A1454" t="inlineStr">
         <is>
-          <t>Asian Market Café</t>
+          <t>Barossa</t>
         </is>
       </c>
       <c r="B1454" t="inlineStr"/>
-      <c r="C1454" t="inlineStr">
-        <is>
-          <t>6431 6156</t>
-        </is>
+      <c r="C1454" t="n">
+        <v>65345188</v>
       </c>
       <c r="D1454" t="inlineStr"/>
       <c r="E1454" t="inlineStr"/>
@@ -29465,12 +29455,14 @@
     <row r="1455">
       <c r="A1455" t="inlineStr">
         <is>
-          <t>Atmosphere Bistro &amp; Bar deal</t>
+          <t>Barraka Bar and Restaurant</t>
         </is>
       </c>
       <c r="B1455" t="inlineStr"/>
-      <c r="C1455" t="n">
-        <v>67024906</v>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>6737 9130</t>
+        </is>
       </c>
       <c r="D1455" t="inlineStr"/>
       <c r="E1455" t="inlineStr"/>
@@ -29478,12 +29470,12 @@
     <row r="1456">
       <c r="A1456" t="inlineStr">
         <is>
-          <t>Awe desserts</t>
+          <t>Batter (My Crepe Escape)</t>
         </is>
       </c>
       <c r="B1456" t="inlineStr"/>
       <c r="C1456" t="n">
-        <v>63377430</v>
+        <v>96266029</v>
       </c>
       <c r="D1456" t="inlineStr"/>
       <c r="E1456" t="inlineStr"/>
@@ -29491,27 +29483,31 @@
     <row r="1457">
       <c r="A1457" t="inlineStr">
         <is>
-          <t>Azabu Sabo</t>
+          <t>Bazuka Cafe Bar</t>
         </is>
       </c>
       <c r="B1457" t="inlineStr"/>
-      <c r="C1457" t="n">
-        <v>94235594</v>
-      </c>
-      <c r="D1457" t="inlineStr"/>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1457" t="inlineStr"/>
     </row>
     <row r="1458">
       <c r="A1458" t="inlineStr">
         <is>
-          <t>Azmi restaurant</t>
+          <t>BBQ Chicken</t>
         </is>
       </c>
       <c r="B1458" t="inlineStr"/>
-      <c r="C1458" t="inlineStr">
-        <is>
-          <t>9428 0203</t>
-        </is>
+      <c r="C1458" t="n">
+        <v>64813310</v>
       </c>
       <c r="D1458" t="inlineStr"/>
       <c r="E1458" t="inlineStr"/>
@@ -29519,7 +29515,7 @@
     <row r="1459">
       <c r="A1459" t="inlineStr">
         <is>
-          <t>Bangrak Thai Kitchen</t>
+          <t>Yakiniquest</t>
         </is>
       </c>
       <c r="B1459" t="inlineStr"/>
@@ -29538,12 +29534,13 @@
     <row r="1460">
       <c r="A1460" t="inlineStr">
         <is>
-          <t>Bao Today</t>
+          <t>BeiShanChuan Spicy Steamboat 
+ Restaurant</t>
         </is>
       </c>
       <c r="B1460" t="inlineStr"/>
       <c r="C1460" t="n">
-        <v>62521074</v>
+        <v>62223880</v>
       </c>
       <c r="D1460" t="inlineStr"/>
       <c r="E1460" t="inlineStr"/>
@@ -29551,12 +29548,12 @@
     <row r="1461">
       <c r="A1461" t="inlineStr">
         <is>
-          <t>Bar-a-Thym</t>
+          <t>Beppu Menkan Dining restaurant</t>
         </is>
       </c>
       <c r="B1461" t="inlineStr"/>
       <c r="C1461" t="n">
-        <v>65572224</v>
+        <v>64380328</v>
       </c>
       <c r="D1461" t="inlineStr"/>
       <c r="E1461" t="inlineStr"/>
@@ -29564,12 +29561,12 @@
     <row r="1462">
       <c r="A1462" t="inlineStr">
         <is>
-          <t>Barcook Bakery</t>
+          <t>BerryLite deal</t>
         </is>
       </c>
       <c r="B1462" t="inlineStr"/>
       <c r="C1462" t="n">
-        <v>64626588</v>
+        <v>67933308</v>
       </c>
       <c r="D1462" t="inlineStr"/>
       <c r="E1462" t="inlineStr"/>
@@ -29577,27 +29574,29 @@
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>Barossa</t>
+          <t>Bing Bian</t>
         </is>
       </c>
       <c r="B1463" t="inlineStr"/>
       <c r="C1463" t="n">
-        <v>65345188</v>
-      </c>
-      <c r="D1463" t="inlineStr"/>
+        <v>97879255</v>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +65 63389475</t>
+        </is>
+      </c>
       <c r="E1463" t="inlineStr"/>
     </row>
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>Barraka Bar and Restaurant</t>
+          <t>Bikaner Express</t>
         </is>
       </c>
       <c r="B1464" t="inlineStr"/>
-      <c r="C1464" t="inlineStr">
-        <is>
-          <t>6737 9130</t>
-        </is>
+      <c r="C1464" t="n">
+        <v>62916190</v>
       </c>
       <c r="D1464" t="inlineStr"/>
       <c r="E1464" t="inlineStr"/>
@@ -29605,44 +29604,40 @@
     <row r="1465">
       <c r="A1465" t="inlineStr">
         <is>
-          <t>Batter (My Crepe Escape)</t>
+          <t>Bincho deal</t>
         </is>
       </c>
       <c r="B1465" t="inlineStr"/>
       <c r="C1465" t="n">
-        <v>96266029</v>
-      </c>
-      <c r="D1465" t="inlineStr"/>
+        <v>64384567</v>
+      </c>
+      <c r="D1465" t="n">
+        <v>90499388</v>
+      </c>
       <c r="E1465" t="inlineStr"/>
     </row>
     <row r="1466">
       <c r="A1466" t="inlineStr">
         <is>
-          <t>Bazuka Cafe Bar</t>
+          <t>Bistecca Tuscan Steakhouse</t>
         </is>
       </c>
       <c r="B1466" t="inlineStr"/>
-      <c r="C1466" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1466" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1466" t="n">
+        <v>67356739</v>
+      </c>
+      <c r="D1466" t="inlineStr"/>
       <c r="E1466" t="inlineStr"/>
     </row>
     <row r="1467">
       <c r="A1467" t="inlineStr">
         <is>
-          <t>BBQ Chicken</t>
+          <t>Bistro</t>
         </is>
       </c>
       <c r="B1467" t="inlineStr"/>
       <c r="C1467" t="n">
-        <v>64813310</v>
+        <v>65465229</v>
       </c>
       <c r="D1467" t="inlineStr"/>
       <c r="E1467" t="inlineStr"/>
@@ -29650,33 +29645,25 @@
     <row r="1468">
       <c r="A1468" t="inlineStr">
         <is>
-          <t>Yakiniquest</t>
+          <t>Onion Restaurant</t>
         </is>
       </c>
       <c r="B1468" t="inlineStr"/>
-      <c r="C1468" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1468" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1468" t="n">
+        <v>67578859</v>
+      </c>
+      <c r="D1468" t="inlineStr"/>
       <c r="E1468" t="inlineStr"/>
     </row>
     <row r="1469">
       <c r="A1469" t="inlineStr">
         <is>
-          <t>Bella Pizza</t>
+          <t>Bistroquet</t>
         </is>
       </c>
       <c r="B1469" t="inlineStr"/>
-      <c r="C1469" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1469" t="n">
+        <v>62732774</v>
       </c>
       <c r="D1469" t="inlineStr"/>
       <c r="E1469" t="inlineStr"/>
@@ -29684,14 +29671,12 @@
     <row r="1470">
       <c r="A1470" t="inlineStr">
         <is>
-          <t>The Benjamins deal</t>
+          <t>Bitters &amp; Love</t>
         </is>
       </c>
       <c r="B1470" t="inlineStr"/>
-      <c r="C1470" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1470" t="n">
+        <v>64381836</v>
       </c>
       <c r="D1470" t="inlineStr"/>
       <c r="E1470" t="inlineStr"/>
@@ -29699,13 +29684,12 @@
     <row r="1471">
       <c r="A1471" t="inlineStr">
         <is>
-          <t>BeiShanChuan Spicy Steamboat 
- Restaurant</t>
+          <t>Black &amp; White Cocktail Bar &amp; Bites</t>
         </is>
       </c>
       <c r="B1471" t="inlineStr"/>
       <c r="C1471" t="n">
-        <v>62223880</v>
+        <v>94471826</v>
       </c>
       <c r="D1471" t="inlineStr"/>
       <c r="E1471" t="inlineStr"/>
@@ -29713,12 +29697,12 @@
     <row r="1472">
       <c r="A1472" t="inlineStr">
         <is>
-          <t>Beppu Menkan Dining restaurant</t>
+          <t>Blackbird Bistro &amp; Bar</t>
         </is>
       </c>
       <c r="B1472" t="inlineStr"/>
       <c r="C1472" t="n">
-        <v>64380328</v>
+        <v>63373448</v>
       </c>
       <c r="D1472" t="inlineStr"/>
       <c r="E1472" t="inlineStr"/>
@@ -29726,70 +29710,68 @@
     <row r="1473">
       <c r="A1473" t="inlineStr">
         <is>
-          <t>BerryLite deal</t>
+          <t>Blowfish Bar &amp; Entertainment</t>
         </is>
       </c>
       <c r="B1473" t="inlineStr"/>
       <c r="C1473" t="n">
-        <v>67933308</v>
-      </c>
-      <c r="D1473" t="inlineStr"/>
+        <v>67362056</v>
+      </c>
+      <c r="D1473" t="n">
+        <v>67376036</v>
+      </c>
       <c r="E1473" t="inlineStr"/>
     </row>
     <row r="1474">
       <c r="A1474" t="inlineStr">
         <is>
-          <t>Bing Bian</t>
+          <t>Bliss Garden Restaurant</t>
         </is>
       </c>
       <c r="B1474" t="inlineStr"/>
       <c r="C1474" t="n">
-        <v>97879255</v>
-      </c>
-      <c r="D1474" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> +65 63389475</t>
-        </is>
-      </c>
+        <v>67891313</v>
+      </c>
+      <c r="D1474" t="inlineStr"/>
       <c r="E1474" t="inlineStr"/>
     </row>
     <row r="1475">
       <c r="A1475" t="inlineStr">
         <is>
-          <t>Bikaner Express</t>
+          <t>Blu Jazz</t>
         </is>
       </c>
       <c r="B1475" t="inlineStr"/>
       <c r="C1475" t="n">
-        <v>62916190</v>
-      </c>
-      <c r="D1475" t="inlineStr"/>
+        <v>91990610</v>
+      </c>
+      <c r="D1475" t="n">
+        <v>62911297</v>
+      </c>
       <c r="E1475" t="inlineStr"/>
     </row>
     <row r="1476">
       <c r="A1476" t="inlineStr">
         <is>
-          <t>Bincho deal</t>
+          <t>Blue Mist</t>
         </is>
       </c>
       <c r="B1476" t="inlineStr"/>
       <c r="C1476" t="n">
-        <v>64384567</v>
-      </c>
-      <c r="D1476" t="n">
-        <v>90499388</v>
-      </c>
+        <v>62201820</v>
+      </c>
+      <c r="D1476" t="inlineStr"/>
       <c r="E1476" t="inlineStr"/>
     </row>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
-          <t>Bistecca Tuscan Steakhouse</t>
+          <t>BOCA deal</t>
         </is>
       </c>
       <c r="B1477" t="inlineStr"/>
       <c r="C1477" t="n">
-        <v>67356739</v>
+        <v>62210132</v>
       </c>
       <c r="D1477" t="inlineStr"/>
       <c r="E1477" t="inlineStr"/>
@@ -29797,12 +29779,12 @@
     <row r="1478">
       <c r="A1478" t="inlineStr">
         <is>
-          <t>Bistro</t>
+          <t>Boiler Room</t>
         </is>
       </c>
       <c r="B1478" t="inlineStr"/>
       <c r="C1478" t="n">
-        <v>65465229</v>
+        <v>62707676</v>
       </c>
       <c r="D1478" t="inlineStr"/>
       <c r="E1478" t="inlineStr"/>
@@ -29810,12 +29792,12 @@
     <row r="1479">
       <c r="A1479" t="inlineStr">
         <is>
-          <t>Onion Restaurant</t>
+          <t>boCHINche deal</t>
         </is>
       </c>
       <c r="B1479" t="inlineStr"/>
       <c r="C1479" t="n">
-        <v>67578859</v>
+        <v>62354990</v>
       </c>
       <c r="D1479" t="inlineStr"/>
       <c r="E1479" t="inlineStr"/>
@@ -29823,25 +29805,27 @@
     <row r="1480">
       <c r="A1480" t="inlineStr">
         <is>
-          <t>Bistroquet</t>
+          <t>Bongo Bar</t>
         </is>
       </c>
       <c r="B1480" t="inlineStr"/>
       <c r="C1480" t="n">
-        <v>62732774</v>
-      </c>
-      <c r="D1480" t="inlineStr"/>
+        <v>67362056</v>
+      </c>
+      <c r="D1480" t="n">
+        <v>67376036</v>
+      </c>
       <c r="E1480" t="inlineStr"/>
     </row>
     <row r="1481">
       <c r="A1481" t="inlineStr">
         <is>
-          <t>Bitters &amp; Love</t>
+          <t>Bonkers Pub</t>
         </is>
       </c>
       <c r="B1481" t="inlineStr"/>
       <c r="C1481" t="n">
-        <v>64381836</v>
+        <v>62263817</v>
       </c>
       <c r="D1481" t="inlineStr"/>
       <c r="E1481" t="inlineStr"/>
@@ -29849,12 +29833,12 @@
     <row r="1482">
       <c r="A1482" t="inlineStr">
         <is>
-          <t>Black &amp; White Cocktail Bar &amp; Bites</t>
+          <t>Bosses Restaurant - Black Society -</t>
         </is>
       </c>
       <c r="B1482" t="inlineStr"/>
       <c r="C1482" t="n">
-        <v>94471826</v>
+        <v>63769740</v>
       </c>
       <c r="D1482" t="inlineStr"/>
       <c r="E1482" t="inlineStr"/>
@@ -29862,12 +29846,12 @@
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
-          <t>Blackbird Bistro &amp; Bar</t>
+          <t>Boruto</t>
         </is>
       </c>
       <c r="B1483" t="inlineStr"/>
       <c r="C1483" t="n">
-        <v>63373448</v>
+        <v>65320418</v>
       </c>
       <c r="D1483" t="inlineStr"/>
       <c r="E1483" t="inlineStr"/>
@@ -29875,27 +29859,25 @@
     <row r="1484">
       <c r="A1484" t="inlineStr">
         <is>
-          <t>Blowfish Bar &amp; Entertainment</t>
+          <t>BOTAK JONE</t>
         </is>
       </c>
       <c r="B1484" t="inlineStr"/>
       <c r="C1484" t="n">
-        <v>67362056</v>
-      </c>
-      <c r="D1484" t="n">
-        <v>67376036</v>
-      </c>
+        <v>62890225</v>
+      </c>
+      <c r="D1484" t="inlineStr"/>
       <c r="E1484" t="inlineStr"/>
     </row>
     <row r="1485">
       <c r="A1485" t="inlineStr">
         <is>
-          <t>Bliss Garden Restaurant</t>
+          <t>Brazil Churrasco</t>
         </is>
       </c>
       <c r="B1485" t="inlineStr"/>
       <c r="C1485" t="n">
-        <v>67891313</v>
+        <v>96572472</v>
       </c>
       <c r="D1485" t="inlineStr"/>
       <c r="E1485" t="inlineStr"/>
@@ -29903,27 +29885,25 @@
     <row r="1486">
       <c r="A1486" t="inlineStr">
         <is>
-          <t>Blu Jazz</t>
+          <t>Bread Street Kitchen</t>
         </is>
       </c>
       <c r="B1486" t="inlineStr"/>
       <c r="C1486" t="n">
-        <v>91990610</v>
-      </c>
-      <c r="D1486" t="n">
-        <v>62911297</v>
-      </c>
+        <v>66885665</v>
+      </c>
+      <c r="D1486" t="inlineStr"/>
       <c r="E1486" t="inlineStr"/>
     </row>
     <row r="1487">
       <c r="A1487" t="inlineStr">
         <is>
-          <t>Blue Mist</t>
+          <t>Breko Cafe deal</t>
         </is>
       </c>
       <c r="B1487" t="inlineStr"/>
       <c r="C1487" t="n">
-        <v>62201820</v>
+        <v>64684424</v>
       </c>
       <c r="D1487" t="inlineStr"/>
       <c r="E1487" t="inlineStr"/>
@@ -29931,12 +29911,12 @@
     <row r="1488">
       <c r="A1488" t="inlineStr">
         <is>
-          <t>BOCA deal</t>
+          <t>Breeks</t>
         </is>
       </c>
       <c r="B1488" t="inlineStr"/>
       <c r="C1488" t="n">
-        <v>62210132</v>
+        <v>67383368</v>
       </c>
       <c r="D1488" t="inlineStr"/>
       <c r="E1488" t="inlineStr"/>
@@ -29944,12 +29924,12 @@
     <row r="1489">
       <c r="A1489" t="inlineStr">
         <is>
-          <t>Boiler Room</t>
+          <t>Bricks and Cubes</t>
         </is>
       </c>
       <c r="B1489" t="inlineStr"/>
       <c r="C1489" t="n">
-        <v>62707676</v>
+        <v>81213157</v>
       </c>
       <c r="D1489" t="inlineStr"/>
       <c r="E1489" t="inlineStr"/>
@@ -29957,12 +29937,12 @@
     <row r="1490">
       <c r="A1490" t="inlineStr">
         <is>
-          <t>boCHINche deal</t>
+          <t>Brew Maison</t>
         </is>
       </c>
       <c r="B1490" t="inlineStr"/>
       <c r="C1490" t="n">
-        <v>62354990</v>
+        <v>86044220</v>
       </c>
       <c r="D1490" t="inlineStr"/>
       <c r="E1490" t="inlineStr"/>
@@ -29970,27 +29950,25 @@
     <row r="1491">
       <c r="A1491" t="inlineStr">
         <is>
-          <t>Bongo Bar</t>
+          <t>Bukang Korean BBQ &amp; Seafood Restaurant</t>
         </is>
       </c>
       <c r="B1491" t="inlineStr"/>
       <c r="C1491" t="n">
-        <v>67362056</v>
-      </c>
-      <c r="D1491" t="n">
-        <v>67376036</v>
-      </c>
+        <v>63274123</v>
+      </c>
+      <c r="D1491" t="inlineStr"/>
       <c r="E1491" t="inlineStr"/>
     </row>
     <row r="1492">
       <c r="A1492" t="inlineStr">
         <is>
-          <t>Bonkers Pub</t>
+          <t>Bulldog Cafe &amp; Pub</t>
         </is>
       </c>
       <c r="B1492" t="inlineStr"/>
       <c r="C1492" t="n">
-        <v>62263817</v>
+        <v>62848984</v>
       </c>
       <c r="D1492" t="inlineStr"/>
       <c r="E1492" t="inlineStr"/>
@@ -29998,25 +29976,27 @@
     <row r="1493">
       <c r="A1493" t="inlineStr">
         <is>
-          <t>Bosses Restaurant - Black Society -</t>
+          <t>Bumbo Rum Club</t>
         </is>
       </c>
       <c r="B1493" t="inlineStr"/>
       <c r="C1493" t="n">
-        <v>63769740</v>
-      </c>
-      <c r="D1493" t="inlineStr"/>
+        <v>66907500</v>
+      </c>
+      <c r="D1493" t="n">
+        <v>66907598</v>
+      </c>
       <c r="E1493" t="inlineStr"/>
     </row>
     <row r="1494">
       <c r="A1494" t="inlineStr">
         <is>
-          <t>Boruto</t>
+          <t>Butter Factory</t>
         </is>
       </c>
       <c r="B1494" t="inlineStr"/>
       <c r="C1494" t="n">
-        <v>65320418</v>
+        <v>93382353</v>
       </c>
       <c r="D1494" t="inlineStr"/>
       <c r="E1494" t="inlineStr"/>
@@ -30024,12 +30004,12 @@
     <row r="1495">
       <c r="A1495" t="inlineStr">
         <is>
-          <t>BOTAK JONE</t>
+          <t>Bene Spaghetti</t>
         </is>
       </c>
       <c r="B1495" t="inlineStr"/>
       <c r="C1495" t="n">
-        <v>62890225</v>
+        <v>65361726</v>
       </c>
       <c r="D1495" t="inlineStr"/>
       <c r="E1495" t="inlineStr"/>
@@ -30037,14 +30017,12 @@
     <row r="1496">
       <c r="A1496" t="inlineStr">
         <is>
-          <t>Boufe deal</t>
+          <t>Bernie's Restaurant &amp; Bar</t>
         </is>
       </c>
       <c r="B1496" t="inlineStr"/>
-      <c r="C1496" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1496" t="n">
+        <v>65422232</v>
       </c>
       <c r="D1496" t="inlineStr"/>
       <c r="E1496" t="inlineStr"/>
@@ -30052,14 +30030,12 @@
     <row r="1497">
       <c r="A1497" t="inlineStr">
         <is>
-          <t>Brandker Group Sdn Bhd</t>
+          <t>Bibigo</t>
         </is>
       </c>
       <c r="B1497" t="inlineStr"/>
-      <c r="C1497" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1497" t="n">
+        <v>97778245</v>
       </c>
       <c r="D1497" t="inlineStr"/>
       <c r="E1497" t="inlineStr"/>
@@ -30067,14 +30043,12 @@
     <row r="1498">
       <c r="A1498" t="inlineStr">
         <is>
-          <t>BRATWORKS The German Imbiss</t>
+          <t>Big boy</t>
         </is>
       </c>
       <c r="B1498" t="inlineStr"/>
-      <c r="C1498" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1498" t="n">
+        <v>91110726</v>
       </c>
       <c r="D1498" t="inlineStr"/>
       <c r="E1498" t="inlineStr"/>
@@ -30082,40 +30056,46 @@
     <row r="1499">
       <c r="A1499" t="inlineStr">
         <is>
-          <t>Brasserie Gavroche</t>
+          <t>BigMama Deal</t>
         </is>
       </c>
       <c r="B1499" t="inlineStr"/>
       <c r="C1499" t="inlineStr">
         <is>
-          <t>#ERROR!</t>
-        </is>
-      </c>
-      <c r="D1499" t="inlineStr"/>
+          <t>9352 2141</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6738 8887 Biopolis</t>
+        </is>
+      </c>
       <c r="E1499" t="inlineStr"/>
     </row>
     <row r="1500">
       <c r="A1500" t="inlineStr">
         <is>
-          <t>Brazil Churrasco</t>
+          <t>Billy Bombers</t>
         </is>
       </c>
       <c r="B1500" t="inlineStr"/>
       <c r="C1500" t="n">
-        <v>96572472</v>
-      </c>
-      <c r="D1500" t="inlineStr"/>
+        <v>94552204</v>
+      </c>
+      <c r="D1500" t="n">
+        <v>66849345</v>
+      </c>
       <c r="E1500" t="inlineStr"/>
     </row>
     <row r="1501">
       <c r="A1501" t="inlineStr">
         <is>
-          <t>Bread Street Kitchen</t>
+          <t>Black Opal</t>
         </is>
       </c>
       <c r="B1501" t="inlineStr"/>
       <c r="C1501" t="n">
-        <v>66885665</v>
+        <v>66816720</v>
       </c>
       <c r="D1501" t="inlineStr"/>
       <c r="E1501" t="inlineStr"/>
@@ -30123,25 +30103,31 @@
     <row r="1502">
       <c r="A1502" t="inlineStr">
         <is>
-          <t>Breko Cafe deal</t>
+          <t>Blue Urban Oasis Llp</t>
         </is>
       </c>
       <c r="B1502" t="inlineStr"/>
-      <c r="C1502" t="n">
-        <v>64684424</v>
-      </c>
-      <c r="D1502" t="inlineStr"/>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1502" t="inlineStr"/>
     </row>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
-          <t>Breeks</t>
+          <t>Bodacious Bar &amp; Bistro</t>
         </is>
       </c>
       <c r="B1503" t="inlineStr"/>
       <c r="C1503" t="n">
-        <v>67383368</v>
+        <v>67789585</v>
       </c>
       <c r="D1503" t="inlineStr"/>
       <c r="E1503" t="inlineStr"/>
@@ -30149,12 +30135,12 @@
     <row r="1504">
       <c r="A1504" t="inlineStr">
         <is>
-          <t>Bricks and Cubes</t>
+          <t>BORNGA Korean</t>
         </is>
       </c>
       <c r="B1504" t="inlineStr"/>
       <c r="C1504" t="n">
-        <v>81213157</v>
+        <v>68363291</v>
       </c>
       <c r="D1504" t="inlineStr"/>
       <c r="E1504" t="inlineStr"/>
@@ -30162,14 +30148,12 @@
     <row r="1505">
       <c r="A1505" t="inlineStr">
         <is>
-          <t>Buckaroo BBQ and Grill</t>
+          <t>Box n Sticks</t>
         </is>
       </c>
       <c r="B1505" t="inlineStr"/>
-      <c r="C1505" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1505" t="n">
+        <v>63417780</v>
       </c>
       <c r="D1505" t="inlineStr"/>
       <c r="E1505" t="inlineStr"/>
@@ -30177,12 +30161,12 @@
     <row r="1506">
       <c r="A1506" t="inlineStr">
         <is>
-          <t>Brew Maison</t>
+          <t>BQ Bar + Dharma's Kebabs</t>
         </is>
       </c>
       <c r="B1506" t="inlineStr"/>
       <c r="C1506" t="n">
-        <v>86044220</v>
+        <v>82500323</v>
       </c>
       <c r="D1506" t="inlineStr"/>
       <c r="E1506" t="inlineStr"/>
@@ -30190,84 +30174,102 @@
     <row r="1507">
       <c r="A1507" t="inlineStr">
         <is>
-          <t>Bukang Korean BBQ &amp; Seafood Restaurant</t>
+          <t>Brian's Bakes</t>
         </is>
       </c>
       <c r="B1507" t="inlineStr"/>
-      <c r="C1507" t="n">
-        <v>63274123</v>
-      </c>
-      <c r="D1507" t="inlineStr"/>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1507" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1507" t="inlineStr"/>
     </row>
     <row r="1508">
       <c r="A1508" t="inlineStr">
         <is>
-          <t>Bulldog Cafe &amp; Pub</t>
+          <t>Bridge Restaurant &amp; Bar</t>
         </is>
       </c>
       <c r="B1508" t="inlineStr"/>
-      <c r="C1508" t="n">
-        <v>62848984</v>
-      </c>
-      <c r="D1508" t="inlineStr"/>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1508" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1508" t="inlineStr"/>
     </row>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
-          <t>Buona Terra</t>
+          <t>British Hainan</t>
         </is>
       </c>
       <c r="B1509" t="inlineStr"/>
       <c r="C1509" t="inlineStr">
         <is>
-          <t>#ERROR!</t>
-        </is>
-      </c>
-      <c r="D1509" t="inlineStr"/>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1509" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1509" t="inlineStr"/>
     </row>
     <row r="1510">
       <c r="A1510" t="inlineStr">
         <is>
-          <t>Bumbo Rum Club</t>
+          <t>BRIX</t>
         </is>
       </c>
       <c r="B1510" t="inlineStr"/>
       <c r="C1510" t="n">
-        <v>66907500</v>
-      </c>
-      <c r="D1510" t="n">
-        <v>66907598</v>
-      </c>
+        <v>67321234</v>
+      </c>
+      <c r="D1510" t="inlineStr"/>
       <c r="E1510" t="inlineStr"/>
     </row>
     <row r="1511">
       <c r="A1511" t="inlineStr">
         <is>
-          <t>Burlamacco deal</t>
+          <t>Buddy Buddy Cheers</t>
         </is>
       </c>
       <c r="B1511" t="inlineStr"/>
       <c r="C1511" t="inlineStr">
         <is>
-          <t>#ERROR!</t>
-        </is>
-      </c>
-      <c r="D1511" t="inlineStr"/>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1511" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1511" t="inlineStr"/>
     </row>
     <row r="1512">
       <c r="A1512" t="inlineStr">
         <is>
-          <t>Burnt Ends</t>
+          <t>Buffet Town</t>
         </is>
       </c>
       <c r="B1512" t="inlineStr"/>
       <c r="C1512" t="inlineStr">
         <is>
-          <t>#ERROR!</t>
+          <t>6238 0525</t>
         </is>
       </c>
       <c r="D1512" t="inlineStr"/>
@@ -30276,12 +30278,12 @@
     <row r="1513">
       <c r="A1513" t="inlineStr">
         <is>
-          <t>Butter Factory</t>
+          <t>Bumbu Restaurant</t>
         </is>
       </c>
       <c r="B1513" t="inlineStr"/>
       <c r="C1513" t="n">
-        <v>93382353</v>
+        <v>63928628</v>
       </c>
       <c r="D1513" t="inlineStr"/>
       <c r="E1513" t="inlineStr"/>
@@ -30289,12 +30291,14 @@
     <row r="1514">
       <c r="A1514" t="inlineStr">
         <is>
-          <t>Bene Spaghetti</t>
+          <t>Buttergrill deal</t>
         </is>
       </c>
       <c r="B1514" t="inlineStr"/>
-      <c r="C1514" t="n">
-        <v>65361726</v>
+      <c r="C1514" t="inlineStr">
+        <is>
+          <t>65 62212354</t>
+        </is>
       </c>
       <c r="D1514" t="inlineStr"/>
       <c r="E1514" t="inlineStr"/>
@@ -30302,12 +30306,12 @@
     <row r="1515">
       <c r="A1515" t="inlineStr">
         <is>
-          <t>Bernie's Restaurant &amp; Bar</t>
+          <t>Buyan</t>
         </is>
       </c>
       <c r="B1515" t="inlineStr"/>
       <c r="C1515" t="n">
-        <v>65422232</v>
+        <v>62237008</v>
       </c>
       <c r="D1515" t="inlineStr"/>
       <c r="E1515" t="inlineStr"/>
@@ -30315,12 +30319,12 @@
     <row r="1516">
       <c r="A1516" t="inlineStr">
         <is>
-          <t>Bibigo</t>
+          <t>Buttercake N Cream</t>
         </is>
       </c>
       <c r="B1516" t="inlineStr"/>
       <c r="C1516" t="n">
-        <v>97778245</v>
+        <v>67773477</v>
       </c>
       <c r="D1516" t="inlineStr"/>
       <c r="E1516" t="inlineStr"/>
@@ -30328,12 +30332,12 @@
     <row r="1517">
       <c r="A1517" t="inlineStr">
         <is>
-          <t>Big boy</t>
+          <t>Cali Cafe &amp; Bar deal</t>
         </is>
       </c>
       <c r="B1517" t="inlineStr"/>
       <c r="C1517" t="n">
-        <v>91110726</v>
+        <v>66849897</v>
       </c>
       <c r="D1517" t="inlineStr"/>
       <c r="E1517" t="inlineStr"/>
@@ -30341,46 +30345,42 @@
     <row r="1518">
       <c r="A1518" t="inlineStr">
         <is>
-          <t>BigMama Deal</t>
+          <t>Butter Studio deal</t>
         </is>
       </c>
       <c r="B1518" t="inlineStr"/>
       <c r="C1518" t="inlineStr">
         <is>
-          <t>9352 2141</t>
-        </is>
-      </c>
-      <c r="D1518" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6738 8887 Biopolis</t>
-        </is>
-      </c>
+          <t>65 6294711</t>
+        </is>
+      </c>
+      <c r="D1518" t="inlineStr"/>
       <c r="E1518" t="inlineStr"/>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
         <is>
-          <t>Billy Bombers</t>
+          <t>Cacio e Pepe Italian Restaurant</t>
         </is>
       </c>
       <c r="B1519" t="inlineStr"/>
       <c r="C1519" t="n">
-        <v>94552204</v>
-      </c>
-      <c r="D1519" t="n">
-        <v>66849345</v>
-      </c>
+        <v>67603534</v>
+      </c>
+      <c r="D1519" t="inlineStr"/>
       <c r="E1519" t="inlineStr"/>
     </row>
     <row r="1520">
       <c r="A1520" t="inlineStr">
         <is>
-          <t>Black Opal</t>
+          <t>Café Etc. deal</t>
         </is>
       </c>
       <c r="B1520" t="inlineStr"/>
-      <c r="C1520" t="n">
-        <v>66816720</v>
+      <c r="C1520" t="inlineStr">
+        <is>
+          <t>65 62562848</t>
+        </is>
       </c>
       <c r="D1520" t="inlineStr"/>
       <c r="E1520" t="inlineStr"/>
@@ -30388,14 +30388,12 @@
     <row r="1521">
       <c r="A1521" t="inlineStr">
         <is>
-          <t>Bliss House Theme Restaurant</t>
+          <t>Cafe Pal Modern Thai</t>
         </is>
       </c>
       <c r="B1521" t="inlineStr"/>
-      <c r="C1521" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1521" t="n">
+        <v>63335400</v>
       </c>
       <c r="D1521" t="inlineStr"/>
       <c r="E1521" t="inlineStr"/>
@@ -30403,31 +30401,27 @@
     <row r="1522">
       <c r="A1522" t="inlineStr">
         <is>
-          <t>Blue Urban Oasis Llp</t>
+          <t>Caffe B</t>
         </is>
       </c>
       <c r="B1522" t="inlineStr"/>
       <c r="C1522" t="inlineStr">
         <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1522" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+          <t>65 62222329</t>
+        </is>
+      </c>
+      <c r="D1522" t="inlineStr"/>
       <c r="E1522" t="inlineStr"/>
     </row>
     <row r="1523">
       <c r="A1523" t="inlineStr">
         <is>
-          <t>Bodacious Bar &amp; Bistro</t>
+          <t>Calle Real</t>
         </is>
       </c>
       <c r="B1523" t="inlineStr"/>
       <c r="C1523" t="n">
-        <v>67789585</v>
+        <v>64433037</v>
       </c>
       <c r="D1523" t="inlineStr"/>
       <c r="E1523" t="inlineStr"/>
@@ -30435,25 +30429,27 @@
     <row r="1524">
       <c r="A1524" t="inlineStr">
         <is>
-          <t>BORNGA Korean</t>
+          <t>Canadian Pizza ( Bedok reservoir )</t>
         </is>
       </c>
       <c r="B1524" t="inlineStr"/>
       <c r="C1524" t="n">
-        <v>68363291</v>
-      </c>
-      <c r="D1524" t="inlineStr"/>
+        <v>64875654</v>
+      </c>
+      <c r="D1524" t="n">
+        <v>96828963</v>
+      </c>
       <c r="E1524" t="inlineStr"/>
     </row>
     <row r="1525">
       <c r="A1525" t="inlineStr">
         <is>
-          <t>Box n Sticks</t>
+          <t>Candlenut</t>
         </is>
       </c>
       <c r="B1525" t="inlineStr"/>
       <c r="C1525" t="n">
-        <v>63417780</v>
+        <v>81214107</v>
       </c>
       <c r="D1525" t="inlineStr"/>
       <c r="E1525" t="inlineStr"/>
@@ -30461,12 +30457,12 @@
     <row r="1526">
       <c r="A1526" t="inlineStr">
         <is>
-          <t>BQ Bar + Dharma's Kebabs</t>
+          <t>Capri by Fraser Changi</t>
         </is>
       </c>
       <c r="B1526" t="inlineStr"/>
       <c r="C1526" t="n">
-        <v>82500323</v>
+        <v>69339833</v>
       </c>
       <c r="D1526" t="inlineStr"/>
       <c r="E1526" t="inlineStr"/>
@@ -30474,14 +30470,12 @@
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
-          <t>Bravery Cafe</t>
+          <t>Canopy Garden Dining</t>
         </is>
       </c>
       <c r="B1527" t="inlineStr"/>
-      <c r="C1527" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1527" t="n">
+        <v>65561533</v>
       </c>
       <c r="D1527" t="inlineStr"/>
       <c r="E1527" t="inlineStr"/>
@@ -30489,69 +30483,52 @@
     <row r="1528">
       <c r="A1528" t="inlineStr">
         <is>
-          <t>Brian's Bakes</t>
+          <t>Captain Leo</t>
         </is>
       </c>
       <c r="B1528" t="inlineStr"/>
-      <c r="C1528" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1528" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1528" t="n">
+        <v>63363932</v>
+      </c>
+      <c r="D1528" t="inlineStr"/>
       <c r="E1528" t="inlineStr"/>
     </row>
     <row r="1529">
       <c r="A1529" t="inlineStr">
         <is>
-          <t>Bridge Restaurant &amp; Bar</t>
+          <t>CARPENTER AND COOK</t>
         </is>
       </c>
       <c r="B1529" t="inlineStr"/>
-      <c r="C1529" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1529" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1529" t="n">
+        <v>6564633648</v>
+      </c>
+      <c r="D1529" t="inlineStr"/>
       <c r="E1529" t="inlineStr"/>
     </row>
     <row r="1530">
       <c r="A1530" t="inlineStr">
         <is>
-          <t>British Hainan</t>
+          <t>Carvers &amp; Co.</t>
         </is>
       </c>
       <c r="B1530" t="inlineStr"/>
-      <c r="C1530" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1530" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1530" t="n">
+        <v>63480448</v>
+      </c>
+      <c r="D1530" t="inlineStr"/>
       <c r="E1530" t="inlineStr"/>
     </row>
     <row r="1531">
       <c r="A1531" t="inlineStr">
         <is>
-          <t>BRIX</t>
+          <t>Carne &amp; Caipirinha | brazilian
+ churrascaria</t>
         </is>
       </c>
       <c r="B1531" t="inlineStr"/>
       <c r="C1531" t="n">
-        <v>67321234</v>
+        <v>64640478</v>
       </c>
       <c r="D1531" t="inlineStr"/>
       <c r="E1531" t="inlineStr"/>
@@ -30559,33 +30536,25 @@
     <row r="1532">
       <c r="A1532" t="inlineStr">
         <is>
-          <t>Buddy Buddy Cheers</t>
+          <t>Catch Beer &amp; Batter</t>
         </is>
       </c>
       <c r="B1532" t="inlineStr"/>
-      <c r="C1532" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1532" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1532" t="n">
+        <v>81117018</v>
+      </c>
+      <c r="D1532" t="inlineStr"/>
       <c r="E1532" t="inlineStr"/>
     </row>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
-          <t>Buffet Town</t>
+          <t>CATO</t>
         </is>
       </c>
       <c r="B1533" t="inlineStr"/>
-      <c r="C1533" t="inlineStr">
-        <is>
-          <t>6238 0525</t>
-        </is>
+      <c r="C1533" t="n">
+        <v>82996434</v>
       </c>
       <c r="D1533" t="inlineStr"/>
       <c r="E1533" t="inlineStr"/>
@@ -30593,12 +30562,12 @@
     <row r="1534">
       <c r="A1534" t="inlineStr">
         <is>
-          <t>Bumbu Restaurant</t>
+          <t>Central HongKong Cafe @ Wheelock</t>
         </is>
       </c>
       <c r="B1534" t="inlineStr"/>
       <c r="C1534" t="n">
-        <v>63928628</v>
+        <v>96755155</v>
       </c>
       <c r="D1534" t="inlineStr"/>
       <c r="E1534" t="inlineStr"/>
@@ -30606,14 +30575,12 @@
     <row r="1535">
       <c r="A1535" t="inlineStr">
         <is>
-          <t>Buttergrill deal</t>
+          <t>CHA CHA CHA Mexican Restaurant deal</t>
         </is>
       </c>
       <c r="B1535" t="inlineStr"/>
-      <c r="C1535" t="inlineStr">
-        <is>
-          <t>65 62212354</t>
-        </is>
+      <c r="C1535" t="n">
+        <v>64621650</v>
       </c>
       <c r="D1535" t="inlineStr"/>
       <c r="E1535" t="inlineStr"/>
@@ -30621,12 +30588,12 @@
     <row r="1536">
       <c r="A1536" t="inlineStr">
         <is>
-          <t>Buyan</t>
+          <t>Chaitime deal</t>
         </is>
       </c>
       <c r="B1536" t="inlineStr"/>
       <c r="C1536" t="n">
-        <v>62237008</v>
+        <v>96988322</v>
       </c>
       <c r="D1536" t="inlineStr"/>
       <c r="E1536" t="inlineStr"/>
@@ -30634,12 +30601,12 @@
     <row r="1537">
       <c r="A1537" t="inlineStr">
         <is>
-          <t>Buttercake N Cream</t>
+          <t>Chang BBQ</t>
         </is>
       </c>
       <c r="B1537" t="inlineStr"/>
       <c r="C1537" t="n">
-        <v>67773477</v>
+        <v>96722729</v>
       </c>
       <c r="D1537" t="inlineStr"/>
       <c r="E1537" t="inlineStr"/>
@@ -30647,12 +30614,12 @@
     <row r="1538">
       <c r="A1538" t="inlineStr">
         <is>
-          <t>Cali Cafe &amp; Bar deal</t>
+          <t>Charcoal Chicken Express</t>
         </is>
       </c>
       <c r="B1538" t="inlineStr"/>
       <c r="C1538" t="n">
-        <v>66849897</v>
+        <v>62221283</v>
       </c>
       <c r="D1538" t="inlineStr"/>
       <c r="E1538" t="inlineStr"/>
@@ -30660,14 +30627,12 @@
     <row r="1539">
       <c r="A1539" t="inlineStr">
         <is>
-          <t>Butter Studio deal</t>
+          <t>Charlie Brown Cafe</t>
         </is>
       </c>
       <c r="B1539" t="inlineStr"/>
-      <c r="C1539" t="inlineStr">
-        <is>
-          <t>65 6294711</t>
-        </is>
+      <c r="C1539" t="n">
+        <v>6565474909</v>
       </c>
       <c r="D1539" t="inlineStr"/>
       <c r="E1539" t="inlineStr"/>
@@ -30675,12 +30640,12 @@
     <row r="1540">
       <c r="A1540" t="inlineStr">
         <is>
-          <t>Cacio e Pepe Italian Restaurant</t>
+          <t>Charlyn's Milk Bar</t>
         </is>
       </c>
       <c r="B1540" t="inlineStr"/>
       <c r="C1540" t="n">
-        <v>67603534</v>
+        <v>92367263</v>
       </c>
       <c r="D1540" t="inlineStr"/>
       <c r="E1540" t="inlineStr"/>
@@ -30688,14 +30653,12 @@
     <row r="1541">
       <c r="A1541" t="inlineStr">
         <is>
-          <t>Café Etc. deal</t>
+          <t>Chat Masala</t>
         </is>
       </c>
       <c r="B1541" t="inlineStr"/>
-      <c r="C1541" t="inlineStr">
-        <is>
-          <t>65 62562848</t>
-        </is>
+      <c r="C1541" t="n">
+        <v>68760570</v>
       </c>
       <c r="D1541" t="inlineStr"/>
       <c r="E1541" t="inlineStr"/>
@@ -30703,12 +30666,12 @@
     <row r="1542">
       <c r="A1542" t="inlineStr">
         <is>
-          <t>Cafe Pal Modern Thai</t>
+          <t>Cheek by Jowl</t>
         </is>
       </c>
       <c r="B1542" t="inlineStr"/>
       <c r="C1542" t="n">
-        <v>63335400</v>
+        <v>62211911</v>
       </c>
       <c r="D1542" t="inlineStr"/>
       <c r="E1542" t="inlineStr"/>
@@ -30716,14 +30679,12 @@
     <row r="1543">
       <c r="A1543" t="inlineStr">
         <is>
-          <t>Caffe B</t>
+          <t>Chef's Table</t>
         </is>
       </c>
       <c r="B1543" t="inlineStr"/>
-      <c r="C1543" t="inlineStr">
-        <is>
-          <t>65 62222329</t>
-        </is>
+      <c r="C1543" t="n">
+        <v>62244188</v>
       </c>
       <c r="D1543" t="inlineStr"/>
       <c r="E1543" t="inlineStr"/>
@@ -30731,12 +30692,12 @@
     <row r="1544">
       <c r="A1544" t="inlineStr">
         <is>
-          <t>Calle Real</t>
+          <t>Chevy's Bar &amp; Bistro</t>
         </is>
       </c>
       <c r="B1544" t="inlineStr"/>
       <c r="C1544" t="n">
-        <v>64433037</v>
+        <v>62979247</v>
       </c>
       <c r="D1544" t="inlineStr"/>
       <c r="E1544" t="inlineStr"/>
@@ -30744,27 +30705,25 @@
     <row r="1545">
       <c r="A1545" t="inlineStr">
         <is>
-          <t>Canadian Pizza ( Bedok reservoir )</t>
+          <t>Cheng's Seafood Village</t>
         </is>
       </c>
       <c r="B1545" t="inlineStr"/>
       <c r="C1545" t="n">
-        <v>64875654</v>
-      </c>
-      <c r="D1545" t="n">
-        <v>96828963</v>
-      </c>
+        <v>68925590</v>
+      </c>
+      <c r="D1545" t="inlineStr"/>
       <c r="E1545" t="inlineStr"/>
     </row>
     <row r="1546">
       <c r="A1546" t="inlineStr">
         <is>
-          <t>Candlenut</t>
+          <t>Chezcake Bistro</t>
         </is>
       </c>
       <c r="B1546" t="inlineStr"/>
       <c r="C1546" t="n">
-        <v>81214107</v>
+        <v>63466466</v>
       </c>
       <c r="D1546" t="inlineStr"/>
       <c r="E1546" t="inlineStr"/>
@@ -30772,25 +30731,29 @@
     <row r="1547">
       <c r="A1547" t="inlineStr">
         <is>
-          <t>Capri by Fraser Changi</t>
+          <t>Chicken Up (SG)</t>
         </is>
       </c>
       <c r="B1547" t="inlineStr"/>
       <c r="C1547" t="n">
-        <v>69339833</v>
-      </c>
-      <c r="D1547" t="inlineStr"/>
+        <v>63271203</v>
+      </c>
+      <c r="D1547" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6481 4495</t>
+        </is>
+      </c>
       <c r="E1547" t="inlineStr"/>
     </row>
     <row r="1548">
       <c r="A1548" t="inlineStr">
         <is>
-          <t>Canopy Garden Dining</t>
+          <t>Chikaranomoto Global Holdings Pte Ltd</t>
         </is>
       </c>
       <c r="B1548" t="inlineStr"/>
       <c r="C1548" t="n">
-        <v>65561533</v>
+        <v>67332426</v>
       </c>
       <c r="D1548" t="inlineStr"/>
       <c r="E1548" t="inlineStr"/>
@@ -30798,12 +30761,14 @@
     <row r="1549">
       <c r="A1549" t="inlineStr">
         <is>
-          <t>Captain Leo</t>
+          <t>Chilli Padi restaurant</t>
         </is>
       </c>
       <c r="B1549" t="inlineStr"/>
-      <c r="C1549" t="n">
-        <v>63363932</v>
+      <c r="C1549" t="inlineStr">
+        <is>
+          <t>62479531 (O)</t>
+        </is>
       </c>
       <c r="D1549" t="inlineStr"/>
       <c r="E1549" t="inlineStr"/>
@@ -30811,14 +30776,12 @@
     <row r="1550">
       <c r="A1550" t="inlineStr">
         <is>
-          <t>Capricci Bar &amp; Restaurant</t>
+          <t>Chin Huat Live Seafood Restaurant</t>
         </is>
       </c>
       <c r="B1550" t="inlineStr"/>
-      <c r="C1550" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+      <c r="C1550" t="n">
+        <v>67757348</v>
       </c>
       <c r="D1550" t="inlineStr"/>
       <c r="E1550" t="inlineStr"/>
@@ -30826,12 +30789,12 @@
     <row r="1551">
       <c r="A1551" t="inlineStr">
         <is>
-          <t>CARPENTER AND COOK</t>
+          <t>China One deal</t>
         </is>
       </c>
       <c r="B1551" t="inlineStr"/>
       <c r="C1551" t="n">
-        <v>6564633648</v>
+        <v>63390280</v>
       </c>
       <c r="D1551" t="inlineStr"/>
       <c r="E1551" t="inlineStr"/>
@@ -30839,12 +30802,12 @@
     <row r="1552">
       <c r="A1552" t="inlineStr">
         <is>
-          <t>Carvers &amp; Co.</t>
+          <t>CHIPPY British Takeaway</t>
         </is>
       </c>
       <c r="B1552" t="inlineStr"/>
       <c r="C1552" t="n">
-        <v>63480448</v>
+        <v>68753472</v>
       </c>
       <c r="D1552" t="inlineStr"/>
       <c r="E1552" t="inlineStr"/>
@@ -30852,13 +30815,12 @@
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
-          <t>Carne &amp; Caipirinha | brazilian
- churrascaria</t>
+          <t>Cho Omakase</t>
         </is>
       </c>
       <c r="B1553" t="inlineStr"/>
       <c r="C1553" t="n">
-        <v>64640478</v>
+        <v>65322098</v>
       </c>
       <c r="D1553" t="inlineStr"/>
       <c r="E1553" t="inlineStr"/>
@@ -30866,12 +30828,12 @@
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>Catch Beer &amp; Batter</t>
+          <t>BUTTERO</t>
         </is>
       </c>
       <c r="B1554" t="inlineStr"/>
       <c r="C1554" t="n">
-        <v>81117018</v>
+        <v>64387737</v>
       </c>
       <c r="D1554" t="inlineStr"/>
       <c r="E1554" t="inlineStr"/>
@@ -30879,64 +30841,90 @@
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>CATO</t>
+          <t>C.A.N. (Christa &amp; Naomi) Cafe</t>
         </is>
       </c>
       <c r="B1555" t="inlineStr"/>
-      <c r="C1555" t="n">
-        <v>82996434</v>
-      </c>
-      <c r="D1555" t="inlineStr"/>
+      <c r="C1555" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1555" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1555" t="inlineStr"/>
     </row>
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>Central HongKong Cafe @ Wheelock</t>
+          <t>CAD Cafe</t>
         </is>
       </c>
       <c r="B1556" t="inlineStr"/>
-      <c r="C1556" t="n">
-        <v>96755155</v>
-      </c>
-      <c r="D1556" t="inlineStr"/>
+      <c r="C1556" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1556" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1556" t="inlineStr"/>
     </row>
     <row r="1557">
       <c r="A1557" t="inlineStr">
         <is>
-          <t>CHA CHA CHA Mexican Restaurant deal</t>
+          <t>Cafe Duomo deal</t>
         </is>
       </c>
       <c r="B1557" t="inlineStr"/>
-      <c r="C1557" t="n">
-        <v>64621650</v>
-      </c>
-      <c r="D1557" t="inlineStr"/>
+      <c r="C1557" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1557" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1557" t="inlineStr"/>
     </row>
     <row r="1558">
       <c r="A1558" t="inlineStr">
         <is>
-          <t>Chaitime deal</t>
+          <t>Cafe Frenzie Bar &amp; Bistro deal</t>
         </is>
       </c>
       <c r="B1558" t="inlineStr"/>
-      <c r="C1558" t="n">
-        <v>96988322</v>
-      </c>
-      <c r="D1558" t="inlineStr"/>
+      <c r="C1558" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1558" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1558" t="inlineStr"/>
     </row>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
-          <t>Chang BBQ</t>
+          <t>Cafe Mondo</t>
         </is>
       </c>
       <c r="B1559" t="inlineStr"/>
-      <c r="C1559" t="n">
-        <v>96722729</v>
+      <c r="C1559" t="inlineStr">
+        <is>
+          <t>65 68847510</t>
+        </is>
       </c>
       <c r="D1559" t="inlineStr"/>
       <c r="E1559" t="inlineStr"/>
@@ -30944,12 +30932,14 @@
     <row r="1560">
       <c r="A1560" t="inlineStr">
         <is>
-          <t>Charcoal Chicken Express</t>
+          <t>California Pizza</t>
         </is>
       </c>
       <c r="B1560" t="inlineStr"/>
-      <c r="C1560" t="n">
-        <v>62221283</v>
+      <c r="C1560" t="inlineStr">
+        <is>
+          <t>65 6836 0110</t>
+        </is>
       </c>
       <c r="D1560" t="inlineStr"/>
       <c r="E1560" t="inlineStr"/>
@@ -30957,12 +30947,12 @@
     <row r="1561">
       <c r="A1561" t="inlineStr">
         <is>
-          <t>Charlie Brown Cafe</t>
+          <t>Central Thai @ Siglap</t>
         </is>
       </c>
       <c r="B1561" t="inlineStr"/>
       <c r="C1561" t="n">
-        <v>6565474909</v>
+        <v>97470454</v>
       </c>
       <c r="D1561" t="inlineStr"/>
       <c r="E1561" t="inlineStr"/>
@@ -30970,12 +30960,12 @@
     <row r="1562">
       <c r="A1562" t="inlineStr">
         <is>
-          <t>Charlyn's Milk Bar</t>
+          <t>Charcoal Thai</t>
         </is>
       </c>
       <c r="B1562" t="inlineStr"/>
       <c r="C1562" t="n">
-        <v>92367263</v>
+        <v>62886260</v>
       </c>
       <c r="D1562" t="inlineStr"/>
       <c r="E1562" t="inlineStr"/>
@@ -30983,51 +30973,69 @@
     <row r="1563">
       <c r="A1563" t="inlineStr">
         <is>
-          <t>Chat Masala</t>
+          <t>Chateau de Chillon</t>
         </is>
       </c>
       <c r="B1563" t="inlineStr"/>
-      <c r="C1563" t="n">
-        <v>68760570</v>
-      </c>
-      <c r="D1563" t="inlineStr"/>
+      <c r="C1563" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1563" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1563" t="inlineStr"/>
     </row>
     <row r="1564">
       <c r="A1564" t="inlineStr">
         <is>
-          <t>Cheek by Jowl</t>
+          <t>Chatters</t>
         </is>
       </c>
       <c r="B1564" t="inlineStr"/>
-      <c r="C1564" t="n">
-        <v>62211911</v>
-      </c>
-      <c r="D1564" t="inlineStr"/>
+      <c r="C1564" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1564" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1564" t="inlineStr"/>
     </row>
     <row r="1565">
       <c r="A1565" t="inlineStr">
         <is>
-          <t>Chef's Table</t>
+          <t>Chen Fu Ji Sing's Sensation Seafood</t>
         </is>
       </c>
       <c r="B1565" t="inlineStr"/>
-      <c r="C1565" t="n">
-        <v>62244188</v>
-      </c>
-      <c r="D1565" t="inlineStr"/>
+      <c r="C1565" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1565" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1565" t="inlineStr"/>
     </row>
     <row r="1566">
       <c r="A1566" t="inlineStr">
         <is>
-          <t>Chevy's Bar &amp; Bistro</t>
+          <t>Cheng's 27</t>
         </is>
       </c>
       <c r="B1566" t="inlineStr"/>
       <c r="C1566" t="n">
-        <v>62979247</v>
+        <v>98474716</v>
       </c>
       <c r="D1566" t="inlineStr"/>
       <c r="E1566" t="inlineStr"/>
@@ -31035,12 +31043,12 @@
     <row r="1567">
       <c r="A1567" t="inlineStr">
         <is>
-          <t>Cheng's Seafood Village</t>
+          <t>Chettinadu New Restaurant</t>
         </is>
       </c>
       <c r="B1567" t="inlineStr"/>
       <c r="C1567" t="n">
-        <v>68925590</v>
+        <v>62917161</v>
       </c>
       <c r="D1567" t="inlineStr"/>
       <c r="E1567" t="inlineStr"/>
@@ -31048,12 +31056,12 @@
     <row r="1568">
       <c r="A1568" t="inlineStr">
         <is>
-          <t>Chezcake Bistro</t>
+          <t>Chewy Junior</t>
         </is>
       </c>
       <c r="B1568" t="inlineStr"/>
       <c r="C1568" t="n">
-        <v>63466466</v>
+        <v>91110726</v>
       </c>
       <c r="D1568" t="inlineStr"/>
       <c r="E1568" t="inlineStr"/>
@@ -31061,16 +31069,18 @@
     <row r="1569">
       <c r="A1569" t="inlineStr">
         <is>
-          <t>Chicken Up (SG)</t>
+          <t>Chicken Clinic</t>
         </is>
       </c>
       <c r="B1569" t="inlineStr"/>
-      <c r="C1569" t="n">
-        <v>63271203</v>
+      <c r="C1569" t="inlineStr">
+        <is>
+          <t>6227 0331</t>
+        </is>
       </c>
       <c r="D1569" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6481 4495</t>
+          <t xml:space="preserve"> 6532 9006</t>
         </is>
       </c>
       <c r="E1569" t="inlineStr"/>
@@ -31078,12 +31088,12 @@
     <row r="1570">
       <c r="A1570" t="inlineStr">
         <is>
-          <t>Chikaranomoto Global Holdings Pte Ltd</t>
+          <t>CHICKENKEN</t>
         </is>
       </c>
       <c r="B1570" t="inlineStr"/>
       <c r="C1570" t="n">
-        <v>67332426</v>
+        <v>91507257</v>
       </c>
       <c r="D1570" t="inlineStr"/>
       <c r="E1570" t="inlineStr"/>
@@ -31091,27 +31101,31 @@
     <row r="1571">
       <c r="A1571" t="inlineStr">
         <is>
-          <t>Chilli Padi restaurant</t>
+          <t>Chihuly Lounge</t>
         </is>
       </c>
       <c r="B1571" t="inlineStr"/>
       <c r="C1571" t="inlineStr">
         <is>
-          <t>62479531 (O)</t>
-        </is>
-      </c>
-      <c r="D1571" t="inlineStr"/>
+          <t>6227 0331</t>
+        </is>
+      </c>
+      <c r="D1571" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6532 9006</t>
+        </is>
+      </c>
       <c r="E1571" t="inlineStr"/>
     </row>
     <row r="1572">
       <c r="A1572" t="inlineStr">
         <is>
-          <t>Chin Huat Live Seafood Restaurant</t>
+          <t>Chikuwa Tei Japanese Restaurant</t>
         </is>
       </c>
       <c r="B1572" t="inlineStr"/>
       <c r="C1572" t="n">
-        <v>67757348</v>
+        <v>67389395</v>
       </c>
       <c r="D1572" t="inlineStr"/>
       <c r="E1572" t="inlineStr"/>
@@ -31119,12 +31133,13 @@
     <row r="1573">
       <c r="A1573" t="inlineStr">
         <is>
-          <t>China One deal</t>
+          <t>Chinese Restaurant Hot
+  Pot</t>
         </is>
       </c>
       <c r="B1573" t="inlineStr"/>
       <c r="C1573" t="n">
-        <v>63390280</v>
+        <v>96473930</v>
       </c>
       <c r="D1573" t="inlineStr"/>
       <c r="E1573" t="inlineStr"/>
@@ -31132,12 +31147,12 @@
     <row r="1574">
       <c r="A1574" t="inlineStr">
         <is>
-          <t>CHIPPY British Takeaway</t>
+          <t>Chock Full of Beans deal</t>
         </is>
       </c>
       <c r="B1574" t="inlineStr"/>
       <c r="C1574" t="n">
-        <v>68753472</v>
+        <v>62148839</v>
       </c>
       <c r="D1574" t="inlineStr"/>
       <c r="E1574" t="inlineStr"/>
@@ -31145,25 +31160,28 @@
     <row r="1575">
       <c r="A1575" t="inlineStr">
         <is>
-          <t>Cho Omakase</t>
+          <t>Chong Qing Grilled Fish</t>
         </is>
       </c>
       <c r="B1575" t="inlineStr"/>
       <c r="C1575" t="n">
-        <v>65322098</v>
-      </c>
-      <c r="D1575" t="inlineStr"/>
+        <v>63339148</v>
+      </c>
+      <c r="D1575" t="n">
+        <v>62250087</v>
+      </c>
       <c r="E1575" t="inlineStr"/>
     </row>
     <row r="1576">
       <c r="A1576" t="inlineStr">
         <is>
-          <t>BUTTERO</t>
+          <t>Chong Qing Zheng Zong Lao Huo 
+ Guo Wang</t>
         </is>
       </c>
       <c r="B1576" t="inlineStr"/>
       <c r="C1576" t="n">
-        <v>64387737</v>
+        <v>63345682</v>
       </c>
       <c r="D1576" t="inlineStr"/>
       <c r="E1576" t="inlineStr"/>
@@ -31171,37 +31189,31 @@
     <row r="1577">
       <c r="A1577" t="inlineStr">
         <is>
-          <t>C.A.N. (Christa &amp; Naomi) Cafe</t>
+          <t>Chupitos Bar</t>
         </is>
       </c>
       <c r="B1577" t="inlineStr"/>
-      <c r="C1577" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1577" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
+      <c r="C1577" t="n">
+        <v>63334513</v>
+      </c>
+      <c r="D1577" t="n">
+        <v>62950017</v>
       </c>
       <c r="E1577" t="inlineStr"/>
     </row>
     <row r="1578">
       <c r="A1578" t="inlineStr">
         <is>
-          <t>CAD Cafe</t>
+          <t>Choupinette</t>
         </is>
       </c>
       <c r="B1578" t="inlineStr"/>
-      <c r="C1578" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
+      <c r="C1578" t="n">
+        <v>64660613</v>
       </c>
       <c r="D1578" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6532 9006</t>
+          <t xml:space="preserve"> ( JASON number -6466 0613)</t>
         </is>
       </c>
       <c r="E1578" t="inlineStr"/>
@@ -31209,52 +31221,38 @@
     <row r="1579">
       <c r="A1579" t="inlineStr">
         <is>
-          <t>Cafe Duomo deal</t>
+          <t>Chopsuey Cafe</t>
         </is>
       </c>
       <c r="B1579" t="inlineStr"/>
-      <c r="C1579" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1579" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1579" t="n">
+        <v>92246611</v>
+      </c>
+      <c r="D1579" t="inlineStr"/>
       <c r="E1579" t="inlineStr"/>
     </row>
     <row r="1580">
       <c r="A1580" t="inlineStr">
         <is>
-          <t>Cafe Frenzie Bar &amp; Bistro deal</t>
+          <t>Chotto Matte deal</t>
         </is>
       </c>
       <c r="B1580" t="inlineStr"/>
-      <c r="C1580" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1580" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1580" t="n">
+        <v>62228846</v>
+      </c>
+      <c r="D1580" t="inlineStr"/>
       <c r="E1580" t="inlineStr"/>
     </row>
     <row r="1581">
       <c r="A1581" t="inlineStr">
         <is>
-          <t>Cafe Mondo</t>
+          <t>Chye Seng Huat Hardware deal</t>
         </is>
       </c>
       <c r="B1581" t="inlineStr"/>
-      <c r="C1581" t="inlineStr">
-        <is>
-          <t>65 68847510</t>
-        </is>
+      <c r="C1581" t="n">
+        <v>63960609</v>
       </c>
       <c r="D1581" t="inlineStr"/>
       <c r="E1581" t="inlineStr"/>
@@ -31262,14 +31260,12 @@
     <row r="1582">
       <c r="A1582" t="inlineStr">
         <is>
-          <t>California Pizza</t>
+          <t>Ciao@ Italian Risto-Bar</t>
         </is>
       </c>
       <c r="B1582" t="inlineStr"/>
-      <c r="C1582" t="inlineStr">
-        <is>
-          <t>65 6836 0110</t>
-        </is>
+      <c r="C1582" t="n">
+        <v>62969688</v>
       </c>
       <c r="D1582" t="inlineStr"/>
       <c r="E1582" t="inlineStr"/>
@@ -31277,12 +31273,12 @@
     <row r="1583">
       <c r="A1583" t="inlineStr">
         <is>
-          <t>Central Thai @ Siglap</t>
+          <t>Citrus House</t>
         </is>
       </c>
       <c r="B1583" t="inlineStr"/>
       <c r="C1583" t="n">
-        <v>97470454</v>
+        <v>65363877</v>
       </c>
       <c r="D1583" t="inlineStr"/>
       <c r="E1583" t="inlineStr"/>
@@ -31290,12 +31286,12 @@
     <row r="1584">
       <c r="A1584" t="inlineStr">
         <is>
-          <t>Charcoal Thai</t>
+          <t>Cicheti deal</t>
         </is>
       </c>
       <c r="B1584" t="inlineStr"/>
       <c r="C1584" t="n">
-        <v>62886260</v>
+        <v>62925012</v>
       </c>
       <c r="D1584" t="inlineStr"/>
       <c r="E1584" t="inlineStr"/>
@@ -31303,37 +31299,31 @@
     <row r="1585">
       <c r="A1585" t="inlineStr">
         <is>
-          <t>Chateau de Chillon</t>
+          <t>Club Meatballs</t>
         </is>
       </c>
       <c r="B1585" t="inlineStr"/>
-      <c r="C1585" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1585" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1585" t="n">
+        <v>62228660</v>
+      </c>
+      <c r="D1585" t="inlineStr"/>
       <c r="E1585" t="inlineStr"/>
     </row>
     <row r="1586">
       <c r="A1586" t="inlineStr">
         <is>
-          <t>Chatters</t>
+          <t>Cluck Cluck @ tanjong pagar</t>
         </is>
       </c>
       <c r="B1586" t="inlineStr"/>
       <c r="C1586" t="inlineStr">
         <is>
-          <t>6227 0331</t>
+          <t>9018 9236</t>
         </is>
       </c>
       <c r="D1586" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6532 9006</t>
+          <t xml:space="preserve"> 9198 2673</t>
         </is>
       </c>
       <c r="E1586" t="inlineStr"/>
@@ -31341,31 +31331,25 @@
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
-          <t>Chen Fu Ji Sing's Sensation Seafood</t>
+          <t>Cocobay Indian Cuisine</t>
         </is>
       </c>
       <c r="B1587" t="inlineStr"/>
-      <c r="C1587" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1587" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1587" t="n">
+        <v>93214858</v>
+      </c>
+      <c r="D1587" t="inlineStr"/>
       <c r="E1587" t="inlineStr"/>
     </row>
     <row r="1588">
       <c r="A1588" t="inlineStr">
         <is>
-          <t>Cheng's 27</t>
+          <t>Club Street Social</t>
         </is>
       </c>
       <c r="B1588" t="inlineStr"/>
       <c r="C1588" t="n">
-        <v>98474716</v>
+        <v>62255043</v>
       </c>
       <c r="D1588" t="inlineStr"/>
       <c r="E1588" t="inlineStr"/>
@@ -31373,12 +31357,14 @@
     <row r="1589">
       <c r="A1589" t="inlineStr">
         <is>
-          <t>Chettinadu New Restaurant</t>
+          <t>Cocotte deal</t>
         </is>
       </c>
       <c r="B1589" t="inlineStr"/>
-      <c r="C1589" t="n">
-        <v>62917161</v>
+      <c r="C1589" t="inlineStr">
+        <is>
+          <t>65 62981188</t>
+        </is>
       </c>
       <c r="D1589" t="inlineStr"/>
       <c r="E1589" t="inlineStr"/>
@@ -31386,12 +31372,12 @@
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>Chewy Junior</t>
+          <t>Coffee Anatomy</t>
         </is>
       </c>
       <c r="B1590" t="inlineStr"/>
       <c r="C1590" t="n">
-        <v>91110726</v>
+        <v>96858187</v>
       </c>
       <c r="D1590" t="inlineStr"/>
       <c r="E1590" t="inlineStr"/>
@@ -31399,31 +31385,27 @@
     <row r="1591">
       <c r="A1591" t="inlineStr">
         <is>
-          <t>Chicken Clinic</t>
+          <t>Coffee Bandits deal</t>
         </is>
       </c>
       <c r="B1591" t="inlineStr"/>
       <c r="C1591" t="inlineStr">
         <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1591" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+          <t>9214 5678</t>
+        </is>
+      </c>
+      <c r="D1591" t="inlineStr"/>
       <c r="E1591" t="inlineStr"/>
     </row>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
-          <t>CHICKENKEN</t>
+          <t>Conclave</t>
         </is>
       </c>
       <c r="B1592" t="inlineStr"/>
       <c r="C1592" t="n">
-        <v>91507257</v>
+        <v>97833892</v>
       </c>
       <c r="D1592" t="inlineStr"/>
       <c r="E1592" t="inlineStr"/>
@@ -31431,327 +31413,15 @@
     <row r="1593">
       <c r="A1593" t="inlineStr">
         <is>
-          <t>Chihuly Lounge</t>
+          <t>Coffee: Nowhere</t>
         </is>
       </c>
       <c r="B1593" t="inlineStr"/>
-      <c r="C1593" t="inlineStr">
-        <is>
-          <t>6227 0331</t>
-        </is>
-      </c>
-      <c r="D1593" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6532 9006</t>
-        </is>
-      </c>
+      <c r="C1593" t="n">
+        <v>96570287</v>
+      </c>
+      <c r="D1593" t="inlineStr"/>
       <c r="E1593" t="inlineStr"/>
-    </row>
-    <row r="1594">
-      <c r="A1594" t="inlineStr">
-        <is>
-          <t>Chikuwa Tei Japanese Restaurant</t>
-        </is>
-      </c>
-      <c r="B1594" t="inlineStr"/>
-      <c r="C1594" t="n">
-        <v>67389395</v>
-      </c>
-      <c r="D1594" t="inlineStr"/>
-      <c r="E1594" t="inlineStr"/>
-    </row>
-    <row r="1595">
-      <c r="A1595" t="inlineStr">
-        <is>
-          <t>Chinese Restaurant Hot
-  Pot</t>
-        </is>
-      </c>
-      <c r="B1595" t="inlineStr"/>
-      <c r="C1595" t="n">
-        <v>96473930</v>
-      </c>
-      <c r="D1595" t="inlineStr"/>
-      <c r="E1595" t="inlineStr"/>
-    </row>
-    <row r="1596">
-      <c r="A1596" t="inlineStr">
-        <is>
-          <t>Chock Full of Beans deal</t>
-        </is>
-      </c>
-      <c r="B1596" t="inlineStr"/>
-      <c r="C1596" t="n">
-        <v>62148839</v>
-      </c>
-      <c r="D1596" t="inlineStr"/>
-      <c r="E1596" t="inlineStr"/>
-    </row>
-    <row r="1597">
-      <c r="A1597" t="inlineStr">
-        <is>
-          <t>Chong Qing Grilled Fish</t>
-        </is>
-      </c>
-      <c r="B1597" t="inlineStr"/>
-      <c r="C1597" t="n">
-        <v>63339148</v>
-      </c>
-      <c r="D1597" t="n">
-        <v>62250087</v>
-      </c>
-      <c r="E1597" t="inlineStr"/>
-    </row>
-    <row r="1598">
-      <c r="A1598" t="inlineStr">
-        <is>
-          <t>Chong Qing Zheng Zong Lao Huo 
- Guo Wang</t>
-        </is>
-      </c>
-      <c r="B1598" t="inlineStr"/>
-      <c r="C1598" t="n">
-        <v>63345682</v>
-      </c>
-      <c r="D1598" t="inlineStr"/>
-      <c r="E1598" t="inlineStr"/>
-    </row>
-    <row r="1599">
-      <c r="A1599" t="inlineStr">
-        <is>
-          <t>Chupitos Bar</t>
-        </is>
-      </c>
-      <c r="B1599" t="inlineStr"/>
-      <c r="C1599" t="n">
-        <v>63334513</v>
-      </c>
-      <c r="D1599" t="n">
-        <v>62950017</v>
-      </c>
-      <c r="E1599" t="inlineStr"/>
-    </row>
-    <row r="1600">
-      <c r="A1600" t="inlineStr">
-        <is>
-          <t>Choupinette</t>
-        </is>
-      </c>
-      <c r="B1600" t="inlineStr"/>
-      <c r="C1600" t="n">
-        <v>64660613</v>
-      </c>
-      <c r="D1600" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> ( JASON number -6466 0613)</t>
-        </is>
-      </c>
-      <c r="E1600" t="inlineStr"/>
-    </row>
-    <row r="1601">
-      <c r="A1601" t="inlineStr">
-        <is>
-          <t>Chopsuey Cafe</t>
-        </is>
-      </c>
-      <c r="B1601" t="inlineStr"/>
-      <c r="C1601" t="n">
-        <v>92246611</v>
-      </c>
-      <c r="D1601" t="inlineStr"/>
-      <c r="E1601" t="inlineStr"/>
-    </row>
-    <row r="1602">
-      <c r="A1602" t="inlineStr">
-        <is>
-          <t>Chotto Matte deal</t>
-        </is>
-      </c>
-      <c r="B1602" t="inlineStr"/>
-      <c r="C1602" t="n">
-        <v>62228846</v>
-      </c>
-      <c r="D1602" t="inlineStr"/>
-      <c r="E1602" t="inlineStr"/>
-    </row>
-    <row r="1603">
-      <c r="A1603" t="inlineStr">
-        <is>
-          <t>Chye Seng Huat Hardware deal</t>
-        </is>
-      </c>
-      <c r="B1603" t="inlineStr"/>
-      <c r="C1603" t="n">
-        <v>63960609</v>
-      </c>
-      <c r="D1603" t="inlineStr"/>
-      <c r="E1603" t="inlineStr"/>
-    </row>
-    <row r="1604">
-      <c r="A1604" t="inlineStr">
-        <is>
-          <t>Ciao@ Italian Risto-Bar</t>
-        </is>
-      </c>
-      <c r="B1604" t="inlineStr"/>
-      <c r="C1604" t="n">
-        <v>62969688</v>
-      </c>
-      <c r="D1604" t="inlineStr"/>
-      <c r="E1604" t="inlineStr"/>
-    </row>
-    <row r="1605">
-      <c r="A1605" t="inlineStr">
-        <is>
-          <t>Citrus House</t>
-        </is>
-      </c>
-      <c r="B1605" t="inlineStr"/>
-      <c r="C1605" t="n">
-        <v>65363877</v>
-      </c>
-      <c r="D1605" t="inlineStr"/>
-      <c r="E1605" t="inlineStr"/>
-    </row>
-    <row r="1606">
-      <c r="A1606" t="inlineStr">
-        <is>
-          <t>Cicheti deal</t>
-        </is>
-      </c>
-      <c r="B1606" t="inlineStr"/>
-      <c r="C1606" t="n">
-        <v>62925012</v>
-      </c>
-      <c r="D1606" t="inlineStr"/>
-      <c r="E1606" t="inlineStr"/>
-    </row>
-    <row r="1607">
-      <c r="A1607" t="inlineStr">
-        <is>
-          <t>Club Meatballs</t>
-        </is>
-      </c>
-      <c r="B1607" t="inlineStr"/>
-      <c r="C1607" t="n">
-        <v>62228660</v>
-      </c>
-      <c r="D1607" t="inlineStr"/>
-      <c r="E1607" t="inlineStr"/>
-    </row>
-    <row r="1608">
-      <c r="A1608" t="inlineStr">
-        <is>
-          <t>Cluck Cluck @ tanjong pagar</t>
-        </is>
-      </c>
-      <c r="B1608" t="inlineStr"/>
-      <c r="C1608" t="inlineStr">
-        <is>
-          <t>9018 9236</t>
-        </is>
-      </c>
-      <c r="D1608" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 9198 2673</t>
-        </is>
-      </c>
-      <c r="E1608" t="inlineStr"/>
-    </row>
-    <row r="1609">
-      <c r="A1609" t="inlineStr">
-        <is>
-          <t>Cocobay Indian Cuisine</t>
-        </is>
-      </c>
-      <c r="B1609" t="inlineStr"/>
-      <c r="C1609" t="n">
-        <v>93214858</v>
-      </c>
-      <c r="D1609" t="inlineStr"/>
-      <c r="E1609" t="inlineStr"/>
-    </row>
-    <row r="1610">
-      <c r="A1610" t="inlineStr">
-        <is>
-          <t>Club Street Social</t>
-        </is>
-      </c>
-      <c r="B1610" t="inlineStr"/>
-      <c r="C1610" t="n">
-        <v>62255043</v>
-      </c>
-      <c r="D1610" t="inlineStr"/>
-      <c r="E1610" t="inlineStr"/>
-    </row>
-    <row r="1611">
-      <c r="A1611" t="inlineStr">
-        <is>
-          <t>Cocotte deal</t>
-        </is>
-      </c>
-      <c r="B1611" t="inlineStr"/>
-      <c r="C1611" t="inlineStr">
-        <is>
-          <t>65 62981188</t>
-        </is>
-      </c>
-      <c r="D1611" t="inlineStr"/>
-      <c r="E1611" t="inlineStr"/>
-    </row>
-    <row r="1612">
-      <c r="A1612" t="inlineStr">
-        <is>
-          <t>Coffee Anatomy</t>
-        </is>
-      </c>
-      <c r="B1612" t="inlineStr"/>
-      <c r="C1612" t="n">
-        <v>96858187</v>
-      </c>
-      <c r="D1612" t="inlineStr"/>
-      <c r="E1612" t="inlineStr"/>
-    </row>
-    <row r="1613">
-      <c r="A1613" t="inlineStr">
-        <is>
-          <t>Coffee Bandits deal</t>
-        </is>
-      </c>
-      <c r="B1613" t="inlineStr"/>
-      <c r="C1613" t="inlineStr">
-        <is>
-          <t>9214 5678</t>
-        </is>
-      </c>
-      <c r="D1613" t="inlineStr"/>
-      <c r="E1613" t="inlineStr"/>
-    </row>
-    <row r="1614">
-      <c r="A1614" t="inlineStr">
-        <is>
-          <t>Conclave</t>
-        </is>
-      </c>
-      <c r="B1614" t="inlineStr"/>
-      <c r="C1614" t="n">
-        <v>97833892</v>
-      </c>
-      <c r="D1614" t="inlineStr"/>
-      <c r="E1614" t="inlineStr"/>
-    </row>
-    <row r="1615">
-      <c r="A1615" t="inlineStr">
-        <is>
-          <t>Coffee: Nowhere</t>
-        </is>
-      </c>
-      <c r="B1615" t="inlineStr"/>
-      <c r="C1615" t="n">
-        <v>96570287</v>
-      </c>
-      <c r="D1615" t="inlineStr"/>
-      <c r="E1615" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>